<commit_message>
Fix serial-run failures: raise Playwright test timeout to 30min (was 30s default, caused page/context teardown on long KDF workflows); add pageLORENZO.tab_MyWork (case fix); login-submit step Page pageHome->pageLogin across 33 test cases; add failure-analysis + login-fix scripts
</commit_message>
<xml_diff>
--- a/lorenzo-playwright-kdf/excelFramework/testcases/APE/LSTP_APE_WF001.xlsx
+++ b/lorenzo-playwright-kdf/excelFramework/testcases/APE/LSTP_APE_WF001.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dbashyam2\ORBIS PAS UKI-LZO\ORBIS PAS UKI-LZO\ORBIS PAS UKI-LZO\lorenzo-playwright-kdf\excelFramework\testcases\APE\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bkrishnan6\ORBIS PAS UKI-LZO\lorenzo-playwright-kdf\excelFramework\testcases\APE\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{028BE9B9-1876-45E5-A4EA-303336F9D380}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{25D53D87-9BA3-4528-BFAF-6CB87C6EF1F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{52C8395E-6A7C-4340-B875-65EC1239B4FD}"/>
+    <workbookView xWindow="-120" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{52C8395E-6A7C-4340-B875-65EC1239B4FD}"/>
   </bookViews>
   <sheets>
     <sheet name="TestExecution" sheetId="1" r:id="rId1"/>
@@ -1796,7 +1796,7 @@
         <v>408</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D4" s="6" t="s">
         <v>409</v>
@@ -5370,4 +5370,10 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
+<clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
+  <clbl:label id="{a4153a30-97aa-49dd-8839-66f72081522c}" enabled="1" method="Standard" siteId="{9ffff5c3-bdfa-4a9d-b595-ff68329945ef}" contentBits="0" removed="0"/>
+</clbl:labelList>
 </file>
</xml_diff>

<commit_message>
Add missing 'Find record' (pageHome.lnkTaskPanePatient) step to APE/CarePlan/Charts/Contacts/Observations so the surname field (//input[@dikey='itxtSurname'], verified live) is reachable; StepNo renumbered. Fixes txt_Surname cluster
</commit_message>
<xml_diff>
--- a/lorenzo-playwright-kdf/excelFramework/testcases/APE/LSTP_APE_WF001.xlsx
+++ b/lorenzo-playwright-kdf/excelFramework/testcases/APE/LSTP_APE_WF001.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bkrishnan6\ORBIS PAS UKI-LZO\lorenzo-playwright-kdf\excelFramework\testcases\APE\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{25D53D87-9BA3-4528-BFAF-6CB87C6EF1F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3273DFEC-3092-46A9-9842-3B45F617F8B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{52C8395E-6A7C-4340-B875-65EC1239B4FD}"/>
+    <workbookView xWindow="2775" yWindow="3780" windowWidth="21600" windowHeight="12645" xr2:uid="{52C8395E-6A7C-4340-B875-65EC1239B4FD}"/>
   </bookViews>
   <sheets>
     <sheet name="TestExecution" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="839" uniqueCount="410">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="843" uniqueCount="412">
   <si>
     <t>StepNo</t>
   </si>
@@ -1269,6 +1269,12 @@
   </si>
   <si>
     <t>btn_Login</t>
+  </si>
+  <si>
+    <t>Click Find record to open the patient search form</t>
+  </si>
+  <si>
+    <t>lnkTaskPanePatient</t>
   </si>
 </sst>
 </file>
@@ -1687,7 +1693,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D69C999A-2E1B-4D3F-9F03-720C99658D84}">
-  <dimension ref="A1:K178"/>
+  <dimension ref="A1:K179"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="7.7109375" bestFit="1" customWidth="1"/>
@@ -1813,7 +1819,7 @@
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B5" t="s">
         <v>15</v>
@@ -1830,7 +1836,7 @@
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B6" t="s">
         <v>18</v>
@@ -1844,519 +1850,516 @@
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>19</v>
+        <v>410</v>
+      </c>
+      <c r="C7" t="s">
+        <v>12</v>
+      </c>
+      <c r="D7" t="s">
+        <v>411</v>
       </c>
       <c r="F7" t="s">
-        <v>20</v>
-      </c>
-      <c r="J7" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>22</v>
-      </c>
-      <c r="C8" t="s">
-        <v>23</v>
-      </c>
-      <c r="D8" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="F8" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="J8" t="s">
-        <v>26</v>
+        <v>21</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="C9" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="D9" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="F9" t="s">
-        <v>17</v>
+        <v>25</v>
+      </c>
+      <c r="J9" t="s">
+        <v>26</v>
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="C10" t="s">
-        <v>23</v>
+        <v>28</v>
+      </c>
+      <c r="D10" t="s">
+        <v>29</v>
       </c>
       <c r="F10" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C11" t="s">
-        <v>32</v>
-      </c>
-      <c r="D11" t="s">
-        <v>33</v>
-      </c>
-      <c r="E11" t="s">
-        <v>34</v>
+        <v>23</v>
       </c>
       <c r="F11" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="C12" t="s">
-        <v>36</v>
+        <v>32</v>
+      </c>
+      <c r="D12" t="s">
+        <v>33</v>
+      </c>
+      <c r="E12" t="s">
+        <v>34</v>
       </c>
       <c r="F12" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="C13" t="s">
         <v>36</v>
       </c>
-      <c r="D13" t="s">
-        <v>38</v>
-      </c>
       <c r="F13" t="s">
-        <v>25</v>
-      </c>
-      <c r="K13" t="s">
-        <v>39</v>
+        <v>13</v>
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B14" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="C14" t="s">
         <v>36</v>
       </c>
       <c r="D14" t="s">
-        <v>24</v>
+        <v>38</v>
       </c>
       <c r="F14" t="s">
         <v>25</v>
       </c>
-      <c r="J14" t="s">
-        <v>26</v>
+      <c r="K14" t="s">
+        <v>39</v>
       </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C15" t="s">
         <v>36</v>
       </c>
       <c r="D15" t="s">
-        <v>42</v>
+        <v>24</v>
       </c>
       <c r="F15" t="s">
         <v>25</v>
       </c>
-      <c r="K15" t="s">
-        <v>43</v>
+      <c r="J15" t="s">
+        <v>26</v>
       </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B16" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="C16" t="s">
         <v>36</v>
       </c>
       <c r="D16" t="s">
-        <v>29</v>
+        <v>42</v>
       </c>
       <c r="F16" t="s">
-        <v>17</v>
+        <v>25</v>
+      </c>
+      <c r="K16" t="s">
+        <v>43</v>
       </c>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B17" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C17" t="s">
         <v>36</v>
       </c>
+      <c r="D17" t="s">
+        <v>29</v>
+      </c>
       <c r="F17" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B18" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C18" t="s">
         <v>36</v>
       </c>
-      <c r="D18" t="s">
-        <v>47</v>
-      </c>
       <c r="F18" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B19" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="C19" t="s">
         <v>36</v>
       </c>
       <c r="D19" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="F19" t="s">
-        <v>25</v>
-      </c>
-      <c r="K19" t="s">
-        <v>50</v>
+        <v>17</v>
       </c>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B20" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="C20" t="s">
         <v>36</v>
       </c>
       <c r="D20" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="F20" t="s">
-        <v>53</v>
+        <v>25</v>
       </c>
       <c r="K20" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A21">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B21" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="C21" t="s">
         <v>36</v>
       </c>
       <c r="D21" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="F21" t="s">
-        <v>25</v>
+        <v>53</v>
       </c>
       <c r="K21" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A22">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B22" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="C22" t="s">
         <v>36</v>
       </c>
       <c r="D22" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="F22" t="s">
         <v>25</v>
       </c>
       <c r="K22" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A23">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B23" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="C23" t="s">
         <v>36</v>
       </c>
       <c r="D23" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="F23" t="s">
         <v>25</v>
       </c>
       <c r="K23" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A24">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B24" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="C24" t="s">
         <v>36</v>
       </c>
       <c r="D24" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="F24" t="s">
-        <v>17</v>
+        <v>25</v>
+      </c>
+      <c r="K24" t="s">
+        <v>63</v>
       </c>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A25">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B25" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="C25" t="s">
         <v>36</v>
       </c>
+      <c r="D25" t="s">
+        <v>65</v>
+      </c>
       <c r="F25" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A26">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B26" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C26" t="s">
         <v>36</v>
       </c>
-      <c r="D26" t="s">
-        <v>68</v>
-      </c>
       <c r="F26" t="s">
-        <v>53</v>
-      </c>
-      <c r="K26" t="s">
-        <v>69</v>
+        <v>13</v>
       </c>
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A27">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B27" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="C27" t="s">
         <v>36</v>
       </c>
       <c r="D27" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="F27" t="s">
         <v>53</v>
       </c>
       <c r="K27" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A28">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B28" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="C28" t="s">
         <v>36</v>
       </c>
       <c r="D28" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="F28" t="s">
         <v>53</v>
       </c>
       <c r="K28" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A29">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B29" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="C29" t="s">
         <v>36</v>
       </c>
       <c r="D29" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="F29" t="s">
         <v>53</v>
       </c>
       <c r="K29" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A30">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B30" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="C30" t="s">
         <v>36</v>
       </c>
       <c r="D30" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="F30" t="s">
         <v>53</v>
       </c>
       <c r="K30" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A31">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B31" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="C31" t="s">
         <v>36</v>
       </c>
       <c r="D31" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="F31" t="s">
         <v>53</v>
       </c>
       <c r="K31" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A32">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B32" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="C32" t="s">
         <v>36</v>
       </c>
       <c r="D32" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="F32" t="s">
-        <v>17</v>
+        <v>53</v>
+      </c>
+      <c r="K32" t="s">
+        <v>84</v>
       </c>
     </row>
     <row r="33" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A33">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B33" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="C33" t="s">
-        <v>88</v>
+        <v>36</v>
+      </c>
+      <c r="D33" t="s">
+        <v>86</v>
       </c>
       <c r="F33" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
     </row>
     <row r="34" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A34">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B34" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="C34" t="s">
         <v>88</v>
       </c>
-      <c r="D34" t="s">
-        <v>90</v>
-      </c>
       <c r="F34" t="s">
-        <v>91</v>
-      </c>
-      <c r="J34" t="s">
-        <v>92</v>
+        <v>13</v>
       </c>
     </row>
     <row r="35" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A35">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B35" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="C35" t="s">
         <v>88</v>
@@ -2365,205 +2368,199 @@
         <v>90</v>
       </c>
       <c r="F35" t="s">
-        <v>94</v>
-      </c>
-      <c r="G35" t="s">
-        <v>95</v>
-      </c>
-      <c r="H35" t="s">
-        <v>96</v>
+        <v>91</v>
+      </c>
+      <c r="J35" t="s">
+        <v>92</v>
       </c>
     </row>
     <row r="36" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A36">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B36" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="C36" t="s">
         <v>88</v>
       </c>
       <c r="D36" t="s">
-        <v>98</v>
+        <v>90</v>
       </c>
       <c r="F36" t="s">
-        <v>17</v>
+        <v>94</v>
+      </c>
+      <c r="G36" t="s">
+        <v>95</v>
+      </c>
+      <c r="H36" t="s">
+        <v>96</v>
       </c>
     </row>
     <row r="37" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A37">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B37" t="s">
-        <v>99</v>
+        <v>97</v>
+      </c>
+      <c r="C37" t="s">
+        <v>88</v>
+      </c>
+      <c r="D37" t="s">
+        <v>98</v>
       </c>
       <c r="F37" t="s">
-        <v>14</v>
-      </c>
-      <c r="J37">
-        <v>1</v>
+        <v>17</v>
       </c>
     </row>
     <row r="38" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A38">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B38" t="s">
-        <v>100</v>
-      </c>
-      <c r="C38" t="s">
-        <v>12</v>
+        <v>99</v>
       </c>
       <c r="F38" t="s">
-        <v>13</v>
+        <v>14</v>
+      </c>
+      <c r="J38">
+        <v>1</v>
       </c>
     </row>
     <row r="39" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A39">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B39" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C39" t="s">
         <v>12</v>
       </c>
-      <c r="D39" t="s">
-        <v>102</v>
-      </c>
       <c r="F39" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
     </row>
     <row r="40" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A40">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B40" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="C40" t="s">
-        <v>104</v>
+        <v>12</v>
+      </c>
+      <c r="D40" t="s">
+        <v>102</v>
       </c>
       <c r="F40" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
     </row>
     <row r="41" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A41">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B41" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="C41" t="s">
         <v>104</v>
       </c>
-      <c r="D41" t="s">
-        <v>24</v>
-      </c>
       <c r="F41" t="s">
-        <v>25</v>
-      </c>
-      <c r="J41" t="s">
-        <v>26</v>
+        <v>13</v>
       </c>
     </row>
     <row r="42" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A42">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B42" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C42" t="s">
         <v>104</v>
       </c>
       <c r="D42" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="F42" t="s">
-        <v>17</v>
+        <v>25</v>
+      </c>
+      <c r="J42" t="s">
+        <v>26</v>
       </c>
     </row>
     <row r="43" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A43">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B43" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C43" t="s">
         <v>104</v>
       </c>
+      <c r="D43" t="s">
+        <v>29</v>
+      </c>
       <c r="F43" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
     </row>
     <row r="44" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A44">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B44" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C44" t="s">
-        <v>109</v>
-      </c>
-      <c r="D44" t="s">
-        <v>110</v>
+        <v>104</v>
       </c>
       <c r="F44" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
     </row>
     <row r="45" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A45">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B45" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="C45" t="s">
-        <v>112</v>
+        <v>109</v>
+      </c>
+      <c r="D45" t="s">
+        <v>110</v>
       </c>
       <c r="F45" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
     </row>
     <row r="46" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A46">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B46" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="C46" t="s">
         <v>112</v>
       </c>
-      <c r="D46" t="s">
-        <v>114</v>
-      </c>
       <c r="F46" t="s">
-        <v>94</v>
-      </c>
-      <c r="G46" t="s">
-        <v>115</v>
-      </c>
-      <c r="H46" t="s">
-        <v>116</v>
-      </c>
-      <c r="J46" t="b">
-        <v>1</v>
+        <v>13</v>
       </c>
     </row>
     <row r="47" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A47">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B47" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="C47" t="s">
         <v>112</v>
@@ -2572,665 +2569,674 @@
         <v>114</v>
       </c>
       <c r="F47" t="s">
-        <v>91</v>
-      </c>
-      <c r="J47" t="s">
-        <v>118</v>
+        <v>94</v>
+      </c>
+      <c r="G47" t="s">
+        <v>115</v>
+      </c>
+      <c r="H47" t="s">
+        <v>116</v>
+      </c>
+      <c r="J47" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="48" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A48">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B48" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="C48" t="s">
         <v>112</v>
       </c>
       <c r="D48" t="s">
-        <v>120</v>
+        <v>114</v>
       </c>
       <c r="F48" t="s">
-        <v>17</v>
+        <v>91</v>
+      </c>
+      <c r="J48" t="s">
+        <v>118</v>
       </c>
     </row>
     <row r="49" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A49">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B49" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="C49" t="s">
         <v>112</v>
       </c>
+      <c r="D49" t="s">
+        <v>120</v>
+      </c>
       <c r="F49" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
     </row>
     <row r="50" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A50">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B50" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="C50" t="s">
         <v>112</v>
       </c>
-      <c r="D50" t="s">
-        <v>123</v>
-      </c>
       <c r="F50" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
     </row>
     <row r="51" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A51">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B51" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="C51" t="s">
-        <v>125</v>
+        <v>112</v>
+      </c>
+      <c r="D51" t="s">
+        <v>123</v>
       </c>
       <c r="F51" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
     </row>
     <row r="52" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A52">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B52" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="C52" t="s">
         <v>125</v>
       </c>
-      <c r="D52" t="s">
-        <v>127</v>
-      </c>
       <c r="F52" t="s">
-        <v>53</v>
-      </c>
-      <c r="K52" t="s">
-        <v>128</v>
+        <v>13</v>
       </c>
     </row>
     <row r="53" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A53">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B53" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="C53" t="s">
         <v>125</v>
       </c>
       <c r="D53" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="F53" t="s">
         <v>53</v>
       </c>
       <c r="K53" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
     </row>
     <row r="54" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A54">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B54" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="C54" t="s">
         <v>125</v>
       </c>
       <c r="D54" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="F54" t="s">
         <v>53</v>
       </c>
       <c r="K54" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
     </row>
     <row r="55" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A55">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B55" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="C55" t="s">
         <v>125</v>
       </c>
       <c r="D55" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="F55" t="s">
         <v>53</v>
       </c>
       <c r="K55" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
     </row>
     <row r="56" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A56">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B56" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="C56" t="s">
         <v>125</v>
       </c>
       <c r="D56" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="F56" t="s">
         <v>53</v>
       </c>
       <c r="K56" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
     </row>
     <row r="57" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A57">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B57" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="C57" t="s">
         <v>125</v>
       </c>
       <c r="D57" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="F57" t="s">
-        <v>17</v>
+        <v>53</v>
+      </c>
+      <c r="K57" t="s">
+        <v>140</v>
       </c>
     </row>
     <row r="58" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A58">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B58" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="C58" t="s">
-        <v>144</v>
+        <v>125</v>
+      </c>
+      <c r="D58" t="s">
+        <v>142</v>
       </c>
       <c r="F58" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
     </row>
     <row r="59" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A59">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B59" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="C59" t="s">
         <v>144</v>
       </c>
-      <c r="D59" t="s">
-        <v>146</v>
-      </c>
       <c r="F59" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
     </row>
     <row r="60" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A60">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B60" t="s">
-        <v>147</v>
+        <v>145</v>
+      </c>
+      <c r="C60" t="s">
+        <v>144</v>
+      </c>
+      <c r="D60" t="s">
+        <v>146</v>
       </c>
       <c r="F60" t="s">
-        <v>14</v>
-      </c>
-      <c r="J60">
-        <v>1</v>
+        <v>17</v>
       </c>
     </row>
     <row r="61" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A61">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B61" t="s">
-        <v>148</v>
-      </c>
-      <c r="C61" t="s">
-        <v>112</v>
+        <v>147</v>
       </c>
       <c r="F61" t="s">
-        <v>13</v>
+        <v>14</v>
+      </c>
+      <c r="J61">
+        <v>1</v>
       </c>
     </row>
     <row r="62" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A62">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B62" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="C62" t="s">
         <v>112</v>
       </c>
-      <c r="D62" t="s">
-        <v>150</v>
-      </c>
       <c r="F62" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
     </row>
     <row r="63" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A63">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B63" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="C63" t="s">
         <v>112</v>
       </c>
+      <c r="D63" t="s">
+        <v>150</v>
+      </c>
       <c r="F63" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
     </row>
     <row r="64" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A64">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B64" t="s">
-        <v>152</v>
+        <v>151</v>
+      </c>
+      <c r="C64" t="s">
+        <v>112</v>
       </c>
       <c r="F64" t="s">
-        <v>14</v>
-      </c>
-      <c r="J64">
-        <v>1</v>
+        <v>13</v>
       </c>
     </row>
     <row r="65" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A65">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B65" t="s">
-        <v>153</v>
-      </c>
-      <c r="C65" t="s">
-        <v>112</v>
-      </c>
-      <c r="D65" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="F65" t="s">
-        <v>17</v>
+        <v>14</v>
+      </c>
+      <c r="J65">
+        <v>1</v>
       </c>
     </row>
     <row r="66" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A66">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B66" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="C66" t="s">
-        <v>156</v>
+        <v>112</v>
+      </c>
+      <c r="D66" t="s">
+        <v>154</v>
       </c>
       <c r="F66" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
     </row>
     <row r="67" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A67">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B67" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="C67" t="s">
         <v>156</v>
       </c>
-      <c r="D67" t="s">
-        <v>158</v>
-      </c>
       <c r="F67" t="s">
-        <v>53</v>
-      </c>
-      <c r="K67" t="s">
-        <v>159</v>
+        <v>13</v>
       </c>
     </row>
     <row r="68" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A68">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B68" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="C68" t="s">
         <v>156</v>
       </c>
       <c r="D68" t="s">
-        <v>65</v>
+        <v>158</v>
       </c>
       <c r="F68" t="s">
-        <v>17</v>
+        <v>53</v>
+      </c>
+      <c r="K68" t="s">
+        <v>159</v>
       </c>
     </row>
     <row r="69" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A69">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B69" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="C69" t="s">
-        <v>162</v>
+        <v>156</v>
+      </c>
+      <c r="D69" t="s">
+        <v>65</v>
       </c>
       <c r="F69" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
     </row>
     <row r="70" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A70">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B70" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="C70" t="s">
         <v>162</v>
       </c>
-      <c r="D70" t="s">
-        <v>164</v>
-      </c>
       <c r="F70" t="s">
-        <v>53</v>
-      </c>
-      <c r="K70" t="s">
-        <v>165</v>
+        <v>13</v>
       </c>
     </row>
     <row r="71" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A71">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B71" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="C71" t="s">
         <v>162</v>
       </c>
       <c r="D71" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="F71" t="s">
         <v>53</v>
       </c>
       <c r="K71" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
     </row>
     <row r="72" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A72">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B72" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="C72" t="s">
         <v>162</v>
       </c>
       <c r="D72" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="F72" t="s">
         <v>53</v>
       </c>
       <c r="K72" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
     </row>
     <row r="73" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A73">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B73" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="C73" t="s">
         <v>162</v>
       </c>
       <c r="D73" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="F73" t="s">
         <v>53</v>
       </c>
       <c r="K73" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
     </row>
     <row r="74" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A74">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B74" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="C74" t="s">
         <v>162</v>
       </c>
       <c r="D74" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="F74" t="s">
         <v>53</v>
       </c>
       <c r="K74" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
     </row>
     <row r="75" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A75">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B75" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="C75" t="s">
         <v>162</v>
       </c>
       <c r="D75" t="s">
-        <v>179</v>
+        <v>176</v>
       </c>
       <c r="F75" t="s">
         <v>53</v>
       </c>
       <c r="K75" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
     </row>
     <row r="76" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A76">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B76" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
       <c r="C76" t="s">
         <v>162</v>
       </c>
       <c r="D76" t="s">
-        <v>65</v>
+        <v>179</v>
       </c>
       <c r="F76" t="s">
-        <v>17</v>
+        <v>53</v>
+      </c>
+      <c r="K76" t="s">
+        <v>180</v>
       </c>
     </row>
     <row r="77" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A77">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B77" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="C77" t="s">
-        <v>183</v>
+        <v>162</v>
+      </c>
+      <c r="D77" t="s">
+        <v>65</v>
       </c>
       <c r="F77" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
     </row>
     <row r="78" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A78">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B78" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="C78" t="s">
         <v>183</v>
       </c>
-      <c r="D78" t="s">
-        <v>185</v>
-      </c>
       <c r="F78" t="s">
-        <v>25</v>
-      </c>
-      <c r="K78" t="s">
-        <v>186</v>
+        <v>13</v>
       </c>
     </row>
     <row r="79" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A79">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B79" t="s">
-        <v>187</v>
+        <v>184</v>
       </c>
       <c r="C79" t="s">
         <v>183</v>
       </c>
       <c r="D79" t="s">
-        <v>188</v>
+        <v>185</v>
       </c>
       <c r="F79" t="s">
-        <v>53</v>
+        <v>25</v>
       </c>
       <c r="K79" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
     </row>
     <row r="80" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A80">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B80" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="C80" t="s">
         <v>183</v>
       </c>
       <c r="D80" t="s">
-        <v>142</v>
+        <v>188</v>
       </c>
       <c r="F80" t="s">
-        <v>17</v>
+        <v>53</v>
+      </c>
+      <c r="K80" t="s">
+        <v>189</v>
       </c>
     </row>
     <row r="81" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A81">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B81" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="C81" t="s">
-        <v>192</v>
+        <v>183</v>
+      </c>
+      <c r="D81" t="s">
+        <v>142</v>
       </c>
       <c r="F81" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
     </row>
     <row r="82" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A82">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B82" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="C82" t="s">
         <v>192</v>
       </c>
-      <c r="D82" t="s">
-        <v>194</v>
-      </c>
       <c r="F82" t="s">
-        <v>94</v>
-      </c>
-      <c r="G82" t="s">
-        <v>115</v>
-      </c>
-      <c r="H82" t="b">
-        <v>1</v>
+        <v>13</v>
       </c>
     </row>
     <row r="83" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A83">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B83" t="s">
-        <v>195</v>
+        <v>193</v>
+      </c>
+      <c r="C83" t="s">
+        <v>192</v>
+      </c>
+      <c r="D83" t="s">
+        <v>194</v>
       </c>
       <c r="F83" t="s">
-        <v>14</v>
-      </c>
-      <c r="J83">
+        <v>94</v>
+      </c>
+      <c r="G83" t="s">
+        <v>115</v>
+      </c>
+      <c r="H83" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="84" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A84">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B84" t="s">
-        <v>196</v>
-      </c>
-      <c r="C84" t="s">
-        <v>192</v>
-      </c>
-      <c r="D84" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="F84" t="s">
-        <v>17</v>
+        <v>14</v>
+      </c>
+      <c r="J84">
+        <v>1</v>
       </c>
     </row>
     <row r="85" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A85">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B85" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="C85" t="s">
         <v>192</v>
       </c>
       <c r="D85" t="s">
-        <v>146</v>
+        <v>194</v>
       </c>
       <c r="F85" t="s">
         <v>17</v>
@@ -3238,186 +3244,186 @@
     </row>
     <row r="86" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A86">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B86" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="C86" t="s">
-        <v>199</v>
+        <v>192</v>
+      </c>
+      <c r="D86" t="s">
+        <v>146</v>
       </c>
       <c r="F86" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
     </row>
     <row r="87" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A87">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B87" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="C87" t="s">
         <v>199</v>
       </c>
-      <c r="D87" t="s">
-        <v>65</v>
-      </c>
       <c r="F87" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
     </row>
     <row r="88" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A88">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B88" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="C88" t="s">
-        <v>202</v>
+        <v>199</v>
+      </c>
+      <c r="D88" t="s">
+        <v>65</v>
       </c>
       <c r="F88" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
     </row>
     <row r="89" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A89">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B89" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="C89" t="s">
         <v>202</v>
       </c>
-      <c r="D89" t="s">
-        <v>176</v>
-      </c>
       <c r="F89" t="s">
-        <v>53</v>
-      </c>
-      <c r="K89" t="s">
-        <v>204</v>
+        <v>13</v>
       </c>
     </row>
     <row r="90" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A90">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B90" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="C90" t="s">
         <v>202</v>
       </c>
       <c r="D90" t="s">
-        <v>179</v>
+        <v>176</v>
       </c>
       <c r="F90" t="s">
         <v>53</v>
       </c>
       <c r="K90" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
     </row>
     <row r="91" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A91">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B91" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="C91" t="s">
         <v>202</v>
       </c>
       <c r="D91" t="s">
-        <v>142</v>
+        <v>179</v>
       </c>
       <c r="F91" t="s">
-        <v>17</v>
+        <v>53</v>
+      </c>
+      <c r="K91" t="s">
+        <v>206</v>
       </c>
     </row>
     <row r="92" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A92">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B92" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="C92" t="s">
-        <v>192</v>
+        <v>202</v>
+      </c>
+      <c r="D92" t="s">
+        <v>142</v>
       </c>
       <c r="F92" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
     </row>
     <row r="93" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A93">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B93" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="C93" t="s">
         <v>192</v>
       </c>
-      <c r="D93" t="s">
-        <v>194</v>
-      </c>
       <c r="F93" t="s">
-        <v>94</v>
-      </c>
-      <c r="G93" t="s">
-        <v>115</v>
-      </c>
-      <c r="H93" t="b">
-        <v>1</v>
+        <v>13</v>
       </c>
     </row>
     <row r="94" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A94">
+        <v>93</v>
+      </c>
+      <c r="B94" t="s">
+        <v>209</v>
+      </c>
+      <c r="C94" t="s">
+        <v>192</v>
+      </c>
+      <c r="D94" t="s">
+        <v>194</v>
+      </c>
+      <c r="F94" t="s">
         <v>94</v>
       </c>
-      <c r="B94" t="s">
-        <v>210</v>
-      </c>
-      <c r="F94" t="s">
-        <v>14</v>
-      </c>
-      <c r="J94">
+      <c r="G94" t="s">
+        <v>115</v>
+      </c>
+      <c r="H94" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="95" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A95">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B95" t="s">
-        <v>211</v>
-      </c>
-      <c r="C95" t="s">
-        <v>192</v>
-      </c>
-      <c r="D95" t="s">
-        <v>194</v>
+        <v>210</v>
       </c>
       <c r="F95" t="s">
-        <v>17</v>
+        <v>14</v>
+      </c>
+      <c r="J95">
+        <v>1</v>
       </c>
     </row>
     <row r="96" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A96">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B96" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="C96" t="s">
         <v>192</v>
       </c>
       <c r="D96" t="s">
-        <v>146</v>
+        <v>194</v>
       </c>
       <c r="F96" t="s">
         <v>17</v>
@@ -3425,271 +3431,271 @@
     </row>
     <row r="97" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A97">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B97" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="C97" t="s">
-        <v>199</v>
+        <v>192</v>
+      </c>
+      <c r="D97" t="s">
+        <v>146</v>
       </c>
       <c r="F97" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
     </row>
     <row r="98" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A98">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B98" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="C98" t="s">
         <v>199</v>
       </c>
-      <c r="D98" t="s">
-        <v>65</v>
-      </c>
       <c r="F98" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
     </row>
     <row r="99" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A99">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B99" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="C99" t="s">
-        <v>202</v>
+        <v>199</v>
+      </c>
+      <c r="D99" t="s">
+        <v>65</v>
       </c>
       <c r="F99" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
     </row>
     <row r="100" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A100">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B100" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="C100" t="s">
         <v>202</v>
       </c>
-      <c r="D100" t="s">
-        <v>176</v>
-      </c>
       <c r="F100" t="s">
-        <v>53</v>
-      </c>
-      <c r="K100" t="s">
-        <v>217</v>
+        <v>13</v>
       </c>
     </row>
     <row r="101" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A101">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B101" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="C101" t="s">
         <v>202</v>
       </c>
       <c r="D101" t="s">
-        <v>179</v>
+        <v>176</v>
       </c>
       <c r="F101" t="s">
         <v>53</v>
       </c>
       <c r="K101" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
     </row>
     <row r="102" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A102">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B102" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="C102" t="s">
         <v>202</v>
       </c>
       <c r="D102" t="s">
-        <v>142</v>
+        <v>179</v>
       </c>
       <c r="F102" t="s">
-        <v>17</v>
+        <v>53</v>
+      </c>
+      <c r="K102" t="s">
+        <v>219</v>
       </c>
     </row>
     <row r="103" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A103">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B103" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="C103" t="s">
-        <v>192</v>
+        <v>202</v>
+      </c>
+      <c r="D103" t="s">
+        <v>142</v>
       </c>
       <c r="F103" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
     </row>
     <row r="104" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A104">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B104" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="C104" t="s">
         <v>192</v>
       </c>
-      <c r="D104" t="s">
-        <v>194</v>
-      </c>
       <c r="F104" t="s">
-        <v>94</v>
-      </c>
-      <c r="G104" t="s">
-        <v>115</v>
-      </c>
-      <c r="H104" t="b">
-        <v>1</v>
+        <v>13</v>
       </c>
     </row>
     <row r="105" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A105">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B105" t="s">
-        <v>223</v>
+        <v>222</v>
+      </c>
+      <c r="C105" t="s">
+        <v>192</v>
+      </c>
+      <c r="D105" t="s">
+        <v>194</v>
       </c>
       <c r="F105" t="s">
-        <v>14</v>
-      </c>
-      <c r="J105">
+        <v>94</v>
+      </c>
+      <c r="G105" t="s">
+        <v>115</v>
+      </c>
+      <c r="H105" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="106" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A106">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B106" t="s">
-        <v>224</v>
-      </c>
-      <c r="C106" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="F106" t="s">
-        <v>13</v>
+        <v>14</v>
+      </c>
+      <c r="J106">
+        <v>1</v>
       </c>
     </row>
     <row r="107" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A107">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B107" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="C107" t="s">
         <v>225</v>
       </c>
-      <c r="D107" t="s">
-        <v>227</v>
-      </c>
       <c r="F107" t="s">
-        <v>53</v>
-      </c>
-      <c r="K107" t="s">
-        <v>228</v>
+        <v>13</v>
       </c>
     </row>
     <row r="108" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A108">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B108" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="C108" t="s">
         <v>225</v>
       </c>
       <c r="D108" t="s">
-        <v>230</v>
+        <v>227</v>
       </c>
       <c r="F108" t="s">
         <v>53</v>
       </c>
       <c r="K108" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
     </row>
     <row r="109" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A109">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B109" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="C109" t="s">
         <v>225</v>
       </c>
       <c r="D109" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
       <c r="F109" t="s">
-        <v>17</v>
+        <v>53</v>
+      </c>
+      <c r="K109" t="s">
+        <v>231</v>
       </c>
     </row>
     <row r="110" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A110">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B110" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="C110" t="s">
         <v>225</v>
       </c>
+      <c r="D110" t="s">
+        <v>233</v>
+      </c>
       <c r="F110" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
     </row>
     <row r="111" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A111">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B111" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="C111" t="s">
         <v>225</v>
       </c>
-      <c r="D111" t="s">
-        <v>236</v>
-      </c>
       <c r="F111" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
     </row>
     <row r="112" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A112">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B112" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="C112" t="s">
         <v>225</v>
       </c>
       <c r="D112" t="s">
-        <v>86</v>
+        <v>236</v>
       </c>
       <c r="F112" t="s">
         <v>17</v>
@@ -3697,169 +3703,169 @@
     </row>
     <row r="113" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A113">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B113" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="C113" t="s">
-        <v>192</v>
+        <v>225</v>
+      </c>
+      <c r="D113" t="s">
+        <v>86</v>
       </c>
       <c r="F113" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
     </row>
     <row r="114" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A114">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B114" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="C114" t="s">
         <v>192</v>
       </c>
-      <c r="D114" t="s">
-        <v>194</v>
-      </c>
       <c r="F114" t="s">
-        <v>94</v>
-      </c>
-      <c r="G114" t="s">
-        <v>115</v>
-      </c>
-      <c r="H114" t="b">
-        <v>1</v>
+        <v>13</v>
       </c>
     </row>
     <row r="115" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A115">
+        <v>114</v>
+      </c>
+      <c r="B115" t="s">
+        <v>239</v>
+      </c>
+      <c r="C115" t="s">
+        <v>192</v>
+      </c>
+      <c r="D115" t="s">
+        <v>194</v>
+      </c>
+      <c r="F115" t="s">
+        <v>94</v>
+      </c>
+      <c r="G115" t="s">
         <v>115</v>
       </c>
-      <c r="B115" t="s">
-        <v>240</v>
-      </c>
-      <c r="F115" t="s">
-        <v>14</v>
-      </c>
-      <c r="J115">
+      <c r="H115" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="116" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A116">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B116" t="s">
-        <v>241</v>
-      </c>
-      <c r="C116" t="s">
-        <v>225</v>
+        <v>240</v>
       </c>
       <c r="F116" t="s">
-        <v>13</v>
+        <v>14</v>
+      </c>
+      <c r="J116">
+        <v>1</v>
       </c>
     </row>
     <row r="117" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A117">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B117" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="C117" t="s">
         <v>225</v>
       </c>
-      <c r="D117" t="s">
-        <v>227</v>
-      </c>
       <c r="F117" t="s">
-        <v>53</v>
-      </c>
-      <c r="K117" t="s">
-        <v>243</v>
+        <v>13</v>
       </c>
     </row>
     <row r="118" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A118">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B118" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="C118" t="s">
         <v>225</v>
       </c>
       <c r="D118" t="s">
-        <v>230</v>
+        <v>227</v>
       </c>
       <c r="F118" t="s">
         <v>53</v>
       </c>
       <c r="K118" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
     </row>
     <row r="119" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A119">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="B119" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="C119" t="s">
         <v>225</v>
       </c>
       <c r="D119" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
       <c r="F119" t="s">
-        <v>17</v>
+        <v>53</v>
+      </c>
+      <c r="K119" t="s">
+        <v>245</v>
       </c>
     </row>
     <row r="120" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A120">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B120" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="C120" t="s">
         <v>225</v>
       </c>
+      <c r="D120" t="s">
+        <v>233</v>
+      </c>
       <c r="F120" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
     </row>
     <row r="121" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A121">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B121" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="C121" t="s">
         <v>225</v>
       </c>
-      <c r="D121" t="s">
-        <v>236</v>
-      </c>
       <c r="F121" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
     </row>
     <row r="122" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A122">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="B122" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="C122" t="s">
         <v>225</v>
       </c>
       <c r="D122" t="s">
-        <v>86</v>
+        <v>236</v>
       </c>
       <c r="F122" t="s">
         <v>17</v>
@@ -3867,398 +3873,398 @@
     </row>
     <row r="123" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A123">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B123" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="C123" t="s">
-        <v>192</v>
+        <v>225</v>
+      </c>
+      <c r="D123" t="s">
+        <v>86</v>
       </c>
       <c r="F123" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
     </row>
     <row r="124" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A124">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B124" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="C124" t="s">
         <v>192</v>
       </c>
-      <c r="D124" t="s">
-        <v>194</v>
-      </c>
       <c r="F124" t="s">
-        <v>94</v>
-      </c>
-      <c r="G124" t="s">
-        <v>115</v>
-      </c>
-      <c r="H124" t="b">
-        <v>1</v>
+        <v>13</v>
       </c>
     </row>
     <row r="125" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A125">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B125" t="s">
-        <v>252</v>
+        <v>251</v>
+      </c>
+      <c r="C125" t="s">
+        <v>192</v>
+      </c>
+      <c r="D125" t="s">
+        <v>194</v>
       </c>
       <c r="F125" t="s">
-        <v>14</v>
-      </c>
-      <c r="J125">
+        <v>94</v>
+      </c>
+      <c r="G125" t="s">
+        <v>115</v>
+      </c>
+      <c r="H125" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="126" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A126">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B126" t="s">
-        <v>253</v>
-      </c>
-      <c r="C126" t="s">
-        <v>254</v>
-      </c>
-      <c r="D126" t="s">
-        <v>255</v>
+        <v>252</v>
       </c>
       <c r="F126" t="s">
-        <v>17</v>
+        <v>14</v>
+      </c>
+      <c r="J126">
+        <v>1</v>
       </c>
     </row>
     <row r="127" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A127">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B127" t="s">
-        <v>256</v>
+        <v>253</v>
       </c>
       <c r="C127" t="s">
-        <v>257</v>
+        <v>254</v>
+      </c>
+      <c r="D127" t="s">
+        <v>255</v>
       </c>
       <c r="F127" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
     </row>
     <row r="128" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A128">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B128" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="C128" t="s">
         <v>257</v>
       </c>
-      <c r="D128" t="s">
-        <v>65</v>
-      </c>
       <c r="F128" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
     </row>
     <row r="129" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A129">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B129" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="C129" t="s">
         <v>257</v>
       </c>
+      <c r="D129" t="s">
+        <v>65</v>
+      </c>
       <c r="F129" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
     </row>
     <row r="130" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A130">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B130" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="C130" t="s">
         <v>257</v>
       </c>
-      <c r="D130" t="s">
-        <v>65</v>
-      </c>
       <c r="F130" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
     </row>
     <row r="131" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A131">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B131" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="C131" t="s">
         <v>257</v>
       </c>
+      <c r="D131" t="s">
+        <v>65</v>
+      </c>
       <c r="F131" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
     </row>
     <row r="132" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A132">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B132" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="C132" t="s">
         <v>257</v>
       </c>
-      <c r="D132" t="s">
-        <v>65</v>
-      </c>
       <c r="F132" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
     </row>
     <row r="133" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A133">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="B133" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="C133" t="s">
-        <v>183</v>
+        <v>257</v>
+      </c>
+      <c r="D133" t="s">
+        <v>65</v>
       </c>
       <c r="F133" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
     </row>
     <row r="134" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A134">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B134" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="C134" t="s">
         <v>183</v>
       </c>
-      <c r="D134" t="s">
-        <v>185</v>
-      </c>
       <c r="F134" t="s">
-        <v>25</v>
-      </c>
-      <c r="K134" t="s">
-        <v>265</v>
+        <v>13</v>
       </c>
     </row>
     <row r="135" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A135">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B135" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
       <c r="C135" t="s">
         <v>183</v>
       </c>
       <c r="D135" t="s">
-        <v>188</v>
+        <v>185</v>
       </c>
       <c r="F135" t="s">
-        <v>53</v>
+        <v>25</v>
       </c>
       <c r="K135" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
     </row>
     <row r="136" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A136">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B136" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="C136" t="s">
         <v>183</v>
       </c>
       <c r="D136" t="s">
-        <v>142</v>
+        <v>188</v>
       </c>
       <c r="F136" t="s">
-        <v>17</v>
+        <v>53</v>
+      </c>
+      <c r="K136" t="s">
+        <v>267</v>
       </c>
     </row>
     <row r="137" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A137">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B137" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="C137" t="s">
-        <v>192</v>
+        <v>183</v>
+      </c>
+      <c r="D137" t="s">
+        <v>142</v>
       </c>
       <c r="F137" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
     </row>
     <row r="138" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A138">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B138" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="C138" t="s">
         <v>192</v>
       </c>
-      <c r="D138" t="s">
-        <v>194</v>
-      </c>
       <c r="F138" t="s">
-        <v>94</v>
-      </c>
-      <c r="G138" t="s">
-        <v>115</v>
-      </c>
-      <c r="H138" t="b">
-        <v>1</v>
+        <v>13</v>
       </c>
     </row>
     <row r="139" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A139">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="B139" t="s">
-        <v>271</v>
+        <v>270</v>
+      </c>
+      <c r="C139" t="s">
+        <v>192</v>
+      </c>
+      <c r="D139" t="s">
+        <v>194</v>
       </c>
       <c r="F139" t="s">
-        <v>14</v>
-      </c>
-      <c r="J139">
+        <v>94</v>
+      </c>
+      <c r="G139" t="s">
+        <v>115</v>
+      </c>
+      <c r="H139" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="140" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A140">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B140" t="s">
-        <v>272</v>
-      </c>
-      <c r="C140" t="s">
-        <v>192</v>
+        <v>271</v>
       </c>
       <c r="F140" t="s">
-        <v>13</v>
+        <v>14</v>
+      </c>
+      <c r="J140">
+        <v>1</v>
       </c>
     </row>
     <row r="141" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A141">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="B141" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="C141" t="s">
         <v>192</v>
       </c>
-      <c r="D141" t="s">
-        <v>146</v>
-      </c>
       <c r="F141" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
     </row>
     <row r="142" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A142">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B142" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="C142" t="s">
         <v>192</v>
       </c>
+      <c r="D142" t="s">
+        <v>146</v>
+      </c>
       <c r="F142" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
     </row>
     <row r="143" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A143">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="B143" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="C143" t="s">
         <v>192</v>
       </c>
-      <c r="D143" t="s">
-        <v>276</v>
-      </c>
       <c r="F143" t="s">
-        <v>94</v>
-      </c>
-      <c r="G143" t="s">
-        <v>115</v>
-      </c>
-      <c r="H143" t="b">
-        <v>1</v>
+        <v>13</v>
       </c>
     </row>
     <row r="144" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A144">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B144" t="s">
-        <v>277</v>
+        <v>275</v>
+      </c>
+      <c r="C144" t="s">
+        <v>192</v>
+      </c>
+      <c r="D144" t="s">
+        <v>276</v>
       </c>
       <c r="F144" t="s">
-        <v>14</v>
-      </c>
-      <c r="J144">
+        <v>94</v>
+      </c>
+      <c r="G144" t="s">
+        <v>115</v>
+      </c>
+      <c r="H144" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="145" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A145">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="B145" t="s">
-        <v>278</v>
-      </c>
-      <c r="C145" t="s">
-        <v>192</v>
-      </c>
-      <c r="D145" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="F145" t="s">
-        <v>17</v>
+        <v>14</v>
+      </c>
+      <c r="J145">
+        <v>1</v>
       </c>
     </row>
     <row r="146" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A146">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="B146" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="C146" t="s">
         <v>192</v>
       </c>
       <c r="D146" t="s">
-        <v>146</v>
+        <v>276</v>
       </c>
       <c r="F146" t="s">
         <v>17</v>
@@ -4266,186 +4272,186 @@
     </row>
     <row r="147" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A147">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="B147" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="C147" t="s">
-        <v>281</v>
+        <v>192</v>
+      </c>
+      <c r="D147" t="s">
+        <v>146</v>
       </c>
       <c r="F147" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
     </row>
     <row r="148" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A148">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B148" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="C148" t="s">
         <v>281</v>
       </c>
-      <c r="D148" t="s">
-        <v>283</v>
-      </c>
       <c r="F148" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
     </row>
     <row r="149" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A149">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="B149" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
       <c r="C149" t="s">
         <v>281</v>
       </c>
       <c r="D149" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
       <c r="F149" t="s">
-        <v>25</v>
-      </c>
-      <c r="K149" t="s">
-        <v>286</v>
+        <v>17</v>
       </c>
     </row>
     <row r="150" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A150">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="B150" t="s">
-        <v>287</v>
+        <v>284</v>
       </c>
       <c r="C150" t="s">
         <v>281</v>
       </c>
       <c r="D150" t="s">
-        <v>288</v>
+        <v>285</v>
       </c>
       <c r="F150" t="s">
-        <v>53</v>
+        <v>25</v>
       </c>
       <c r="K150" t="s">
-        <v>289</v>
+        <v>286</v>
       </c>
     </row>
     <row r="151" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A151">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="B151" t="s">
-        <v>290</v>
+        <v>287</v>
       </c>
       <c r="C151" t="s">
         <v>281</v>
       </c>
       <c r="D151" t="s">
-        <v>291</v>
+        <v>288</v>
       </c>
       <c r="F151" t="s">
-        <v>25</v>
+        <v>53</v>
       </c>
       <c r="K151" t="s">
-        <v>292</v>
+        <v>289</v>
       </c>
     </row>
     <row r="152" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A152">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="B152" t="s">
-        <v>293</v>
+        <v>290</v>
       </c>
       <c r="C152" t="s">
         <v>281</v>
       </c>
       <c r="D152" t="s">
-        <v>294</v>
+        <v>291</v>
       </c>
       <c r="F152" t="s">
-        <v>17</v>
+        <v>25</v>
+      </c>
+      <c r="K152" t="s">
+        <v>292</v>
       </c>
     </row>
     <row r="153" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A153">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="B153" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
       <c r="C153" t="s">
-        <v>296</v>
+        <v>281</v>
+      </c>
+      <c r="D153" t="s">
+        <v>294</v>
       </c>
       <c r="F153" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
     </row>
     <row r="154" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A154">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="B154" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
       <c r="C154" t="s">
         <v>296</v>
       </c>
-      <c r="D154" t="s">
-        <v>298</v>
-      </c>
       <c r="F154" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
     </row>
     <row r="155" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A155">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="B155" t="s">
-        <v>299</v>
+        <v>297</v>
       </c>
       <c r="C155" t="s">
-        <v>300</v>
+        <v>296</v>
+      </c>
+      <c r="D155" t="s">
+        <v>298</v>
       </c>
       <c r="F155" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
     </row>
     <row r="156" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A156">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="B156" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
       <c r="C156" t="s">
         <v>300</v>
       </c>
-      <c r="D156" t="s">
-        <v>233</v>
-      </c>
       <c r="F156" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
     </row>
     <row r="157" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A157">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="B157" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="C157" t="s">
         <v>300</v>
       </c>
       <c r="D157" t="s">
-        <v>86</v>
+        <v>233</v>
       </c>
       <c r="F157" t="s">
         <v>17</v>
@@ -4453,115 +4459,115 @@
     </row>
     <row r="158" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A158">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="B158" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="C158" t="s">
-        <v>192</v>
+        <v>300</v>
+      </c>
+      <c r="D158" t="s">
+        <v>86</v>
       </c>
       <c r="F158" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
     </row>
     <row r="159" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A159">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="B159" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="C159" t="s">
         <v>192</v>
       </c>
-      <c r="D159" t="s">
-        <v>276</v>
-      </c>
       <c r="F159" t="s">
-        <v>94</v>
-      </c>
-      <c r="G159" t="s">
-        <v>115</v>
-      </c>
-      <c r="H159" t="b">
-        <v>1</v>
+        <v>13</v>
       </c>
     </row>
     <row r="160" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A160">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="B160" t="s">
-        <v>305</v>
+        <v>304</v>
+      </c>
+      <c r="C160" t="s">
+        <v>192</v>
+      </c>
+      <c r="D160" t="s">
+        <v>276</v>
       </c>
       <c r="F160" t="s">
-        <v>14</v>
-      </c>
-      <c r="J160">
+        <v>94</v>
+      </c>
+      <c r="G160" t="s">
+        <v>115</v>
+      </c>
+      <c r="H160" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="161" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A161">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B161" t="s">
-        <v>306</v>
-      </c>
-      <c r="C161" t="s">
-        <v>192</v>
-      </c>
-      <c r="D161" t="s">
-        <v>276</v>
+        <v>305</v>
       </c>
       <c r="F161" t="s">
-        <v>17</v>
+        <v>14</v>
+      </c>
+      <c r="J161">
+        <v>1</v>
       </c>
     </row>
     <row r="162" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A162">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="B162" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="C162" t="s">
-        <v>308</v>
+        <v>192</v>
+      </c>
+      <c r="D162" t="s">
+        <v>276</v>
       </c>
       <c r="F162" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
     </row>
     <row r="163" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A163">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B163" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
       <c r="C163" t="s">
         <v>308</v>
       </c>
-      <c r="D163" t="s">
-        <v>310</v>
-      </c>
       <c r="F163" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
     </row>
     <row r="164" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A164">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="B164" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
       <c r="C164" t="s">
         <v>308</v>
       </c>
       <c r="D164" t="s">
-        <v>312</v>
+        <v>310</v>
       </c>
       <c r="F164" t="s">
         <v>17</v>
@@ -4569,236 +4575,253 @@
     </row>
     <row r="165" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A165">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="B165" t="s">
-        <v>313</v>
+        <v>311</v>
       </c>
       <c r="C165" t="s">
-        <v>314</v>
+        <v>308</v>
+      </c>
+      <c r="D165" t="s">
+        <v>312</v>
       </c>
       <c r="F165" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
     </row>
     <row r="166" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A166">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="B166" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
       <c r="C166" t="s">
         <v>314</v>
       </c>
-      <c r="D166" t="s">
-        <v>283</v>
-      </c>
       <c r="F166" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
     </row>
     <row r="167" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A167">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="B167" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="C167" t="s">
-        <v>317</v>
+        <v>314</v>
+      </c>
+      <c r="D167" t="s">
+        <v>283</v>
       </c>
       <c r="F167" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
     </row>
     <row r="168" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A168">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="B168" t="s">
-        <v>318</v>
+        <v>316</v>
       </c>
       <c r="C168" t="s">
         <v>317</v>
       </c>
-      <c r="D168" t="s">
-        <v>65</v>
-      </c>
       <c r="F168" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
     </row>
     <row r="169" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A169">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="B169" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="C169" t="s">
-        <v>320</v>
+        <v>317</v>
+      </c>
+      <c r="D169" t="s">
+        <v>65</v>
       </c>
       <c r="F169" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
     </row>
     <row r="170" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A170">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="B170" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
       <c r="C170" t="s">
         <v>320</v>
       </c>
-      <c r="D170" t="s">
-        <v>322</v>
-      </c>
       <c r="F170" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
     </row>
     <row r="171" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A171">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="B171" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
       <c r="C171" t="s">
         <v>320</v>
       </c>
       <c r="D171" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="F171" t="s">
-        <v>53</v>
-      </c>
-      <c r="K171" t="s">
-        <v>325</v>
+        <v>17</v>
       </c>
     </row>
     <row r="172" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A172">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="B172" t="s">
-        <v>326</v>
+        <v>323</v>
       </c>
       <c r="C172" t="s">
         <v>320</v>
       </c>
       <c r="D172" t="s">
-        <v>167</v>
+        <v>324</v>
       </c>
       <c r="F172" t="s">
         <v>53</v>
       </c>
       <c r="K172" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
     </row>
     <row r="173" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A173">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="B173" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="C173" t="s">
         <v>320</v>
       </c>
       <c r="D173" t="s">
-        <v>142</v>
+        <v>167</v>
       </c>
       <c r="F173" t="s">
-        <v>17</v>
+        <v>53</v>
+      </c>
+      <c r="K173" t="s">
+        <v>327</v>
       </c>
     </row>
     <row r="174" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A174">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="B174" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="C174" t="s">
-        <v>192</v>
+        <v>320</v>
+      </c>
+      <c r="D174" t="s">
+        <v>142</v>
       </c>
       <c r="F174" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
     </row>
     <row r="175" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A175">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B175" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="C175" t="s">
         <v>192</v>
       </c>
-      <c r="D175" t="s">
-        <v>276</v>
-      </c>
       <c r="F175" t="s">
-        <v>94</v>
-      </c>
-      <c r="G175" t="s">
-        <v>115</v>
-      </c>
-      <c r="H175" t="b">
-        <v>1</v>
+        <v>13</v>
       </c>
     </row>
     <row r="176" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A176">
+        <v>175</v>
+      </c>
+      <c r="B176" t="s">
+        <v>330</v>
+      </c>
+      <c r="C176" t="s">
+        <v>192</v>
+      </c>
+      <c r="D176" t="s">
+        <v>276</v>
+      </c>
+      <c r="F176" t="s">
+        <v>94</v>
+      </c>
+      <c r="G176" t="s">
+        <v>115</v>
+      </c>
+      <c r="H176" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="177" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A177">
         <v>176</v>
       </c>
-      <c r="B176" t="s">
+      <c r="B177" t="s">
         <v>331</v>
       </c>
-      <c r="F176" t="s">
+      <c r="F177" t="s">
         <v>14</v>
       </c>
-      <c r="J176">
+      <c r="J177">
         <v>1</v>
       </c>
     </row>
-    <row r="177" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A177">
+    <row r="178" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A178">
         <v>177</v>
       </c>
-      <c r="B177" t="s">
+      <c r="B178" t="s">
         <v>332</v>
-      </c>
-      <c r="C177" t="s">
-        <v>12</v>
-      </c>
-      <c r="D177" t="s">
-        <v>333</v>
-      </c>
-      <c r="F177" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="178" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A178">
-        <v>178</v>
-      </c>
-      <c r="B178" t="s">
-        <v>334</v>
       </c>
       <c r="C178" t="s">
         <v>12</v>
       </c>
       <c r="D178" t="s">
+        <v>333</v>
+      </c>
+      <c r="F178" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="179" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A179">
+        <v>178</v>
+      </c>
+      <c r="B179" t="s">
+        <v>334</v>
+      </c>
+      <c r="C179" t="s">
+        <v>12</v>
+      </c>
+      <c r="D179" t="s">
         <v>335</v>
       </c>
-      <c r="F178" t="s">
+      <c r="F179" t="s">
         <v>17</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix Find-record search Find button: add pageSearchPatient.btn_Find (//td[@class='Cmd_TTE' and normalize-space()='Find'], verified live) and point the 5 tests' search btn_Find step to pageSearchPatient (was pageRoadMapButtons/pagePatientBasicSearch's //button[@title='Click to Find'] which doesn't exist in that form)
</commit_message>
<xml_diff>
--- a/lorenzo-playwright-kdf/excelFramework/testcases/APE/LSTP_APE_WF001.xlsx
+++ b/lorenzo-playwright-kdf/excelFramework/testcases/APE/LSTP_APE_WF001.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bkrishnan6\ORBIS PAS UKI-LZO\lorenzo-playwright-kdf\excelFramework\testcases\APE\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3273DFEC-3092-46A9-9842-3B45F617F8B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{24ABB4BA-5AF8-414B-92D4-203596F7494C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2775" yWindow="3780" windowWidth="21600" windowHeight="12645" xr2:uid="{52C8395E-6A7C-4340-B875-65EC1239B4FD}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{52C8395E-6A7C-4340-B875-65EC1239B4FD}"/>
   </bookViews>
   <sheets>
     <sheet name="TestExecution" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="843" uniqueCount="412">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="843" uniqueCount="411">
   <si>
     <t>StepNo</t>
   </si>
@@ -123,9 +123,6 @@
   </si>
   <si>
     <t>Click Find to search for existing patient records</t>
-  </si>
-  <si>
-    <t>pageRoadMapButtons</t>
   </si>
   <si>
     <t>btn_Find</t>
@@ -1749,13 +1746,13 @@
         <v>1</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="C2" s="6" t="s">
         <v>11</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="E2" s="6"/>
       <c r="F2" s="6" t="s">
@@ -1774,13 +1771,13 @@
         <v>2</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="C3" s="6" t="s">
         <v>11</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="E3" s="6"/>
       <c r="F3" s="6" t="s">
@@ -1790,7 +1787,7 @@
       <c r="H3" s="6"/>
       <c r="I3" s="6"/>
       <c r="J3" s="6" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="K3" s="6"/>
     </row>
@@ -1799,13 +1796,13 @@
         <v>3</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="C4" s="6" t="s">
         <v>11</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="E4" s="6"/>
       <c r="F4" s="6" t="s">
@@ -1853,13 +1850,13 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="C7" t="s">
         <v>12</v>
       </c>
       <c r="D7" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="F7" t="s">
         <v>17</v>
@@ -1907,10 +1904,10 @@
         <v>27</v>
       </c>
       <c r="C10" t="s">
+        <v>23</v>
+      </c>
+      <c r="D10" t="s">
         <v>28</v>
-      </c>
-      <c r="D10" t="s">
-        <v>29</v>
       </c>
       <c r="F10" t="s">
         <v>17</v>
@@ -1921,7 +1918,7 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C11" t="s">
         <v>23</v>
@@ -1935,16 +1932,16 @@
         <v>11</v>
       </c>
       <c r="B12" t="s">
+        <v>30</v>
+      </c>
+      <c r="C12" t="s">
         <v>31</v>
       </c>
-      <c r="C12" t="s">
+      <c r="D12" t="s">
         <v>32</v>
       </c>
-      <c r="D12" t="s">
+      <c r="E12" t="s">
         <v>33</v>
-      </c>
-      <c r="E12" t="s">
-        <v>34</v>
       </c>
       <c r="F12" t="s">
         <v>17</v>
@@ -1955,10 +1952,10 @@
         <v>12</v>
       </c>
       <c r="B13" t="s">
+        <v>34</v>
+      </c>
+      <c r="C13" t="s">
         <v>35</v>
-      </c>
-      <c r="C13" t="s">
-        <v>36</v>
       </c>
       <c r="F13" t="s">
         <v>13</v>
@@ -1969,19 +1966,19 @@
         <v>13</v>
       </c>
       <c r="B14" t="s">
+        <v>36</v>
+      </c>
+      <c r="C14" t="s">
+        <v>35</v>
+      </c>
+      <c r="D14" t="s">
         <v>37</v>
-      </c>
-      <c r="C14" t="s">
-        <v>36</v>
-      </c>
-      <c r="D14" t="s">
-        <v>38</v>
       </c>
       <c r="F14" t="s">
         <v>25</v>
       </c>
       <c r="K14" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.25">
@@ -1989,10 +1986,10 @@
         <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C15" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D15" t="s">
         <v>24</v>
@@ -2009,19 +2006,19 @@
         <v>15</v>
       </c>
       <c r="B16" t="s">
+        <v>40</v>
+      </c>
+      <c r="C16" t="s">
+        <v>35</v>
+      </c>
+      <c r="D16" t="s">
         <v>41</v>
-      </c>
-      <c r="C16" t="s">
-        <v>36</v>
-      </c>
-      <c r="D16" t="s">
-        <v>42</v>
       </c>
       <c r="F16" t="s">
         <v>25</v>
       </c>
       <c r="K16" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.25">
@@ -2029,13 +2026,13 @@
         <v>16</v>
       </c>
       <c r="B17" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C17" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D17" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F17" t="s">
         <v>17</v>
@@ -2046,10 +2043,10 @@
         <v>17</v>
       </c>
       <c r="B18" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C18" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="F18" t="s">
         <v>13</v>
@@ -2060,13 +2057,13 @@
         <v>18</v>
       </c>
       <c r="B19" t="s">
+        <v>45</v>
+      </c>
+      <c r="C19" t="s">
+        <v>35</v>
+      </c>
+      <c r="D19" t="s">
         <v>46</v>
-      </c>
-      <c r="C19" t="s">
-        <v>36</v>
-      </c>
-      <c r="D19" t="s">
-        <v>47</v>
       </c>
       <c r="F19" t="s">
         <v>17</v>
@@ -2077,19 +2074,19 @@
         <v>19</v>
       </c>
       <c r="B20" t="s">
+        <v>47</v>
+      </c>
+      <c r="C20" t="s">
+        <v>35</v>
+      </c>
+      <c r="D20" t="s">
         <v>48</v>
-      </c>
-      <c r="C20" t="s">
-        <v>36</v>
-      </c>
-      <c r="D20" t="s">
-        <v>49</v>
       </c>
       <c r="F20" t="s">
         <v>25</v>
       </c>
       <c r="K20" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.25">
@@ -2097,19 +2094,19 @@
         <v>20</v>
       </c>
       <c r="B21" t="s">
+        <v>50</v>
+      </c>
+      <c r="C21" t="s">
+        <v>35</v>
+      </c>
+      <c r="D21" t="s">
         <v>51</v>
       </c>
-      <c r="C21" t="s">
-        <v>36</v>
-      </c>
-      <c r="D21" t="s">
+      <c r="F21" t="s">
         <v>52</v>
       </c>
-      <c r="F21" t="s">
+      <c r="K21" t="s">
         <v>53</v>
-      </c>
-      <c r="K21" t="s">
-        <v>54</v>
       </c>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.25">
@@ -2117,19 +2114,19 @@
         <v>21</v>
       </c>
       <c r="B22" t="s">
+        <v>54</v>
+      </c>
+      <c r="C22" t="s">
+        <v>35</v>
+      </c>
+      <c r="D22" t="s">
         <v>55</v>
-      </c>
-      <c r="C22" t="s">
-        <v>36</v>
-      </c>
-      <c r="D22" t="s">
-        <v>56</v>
       </c>
       <c r="F22" t="s">
         <v>25</v>
       </c>
       <c r="K22" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.25">
@@ -2137,19 +2134,19 @@
         <v>22</v>
       </c>
       <c r="B23" t="s">
+        <v>57</v>
+      </c>
+      <c r="C23" t="s">
+        <v>35</v>
+      </c>
+      <c r="D23" t="s">
         <v>58</v>
-      </c>
-      <c r="C23" t="s">
-        <v>36</v>
-      </c>
-      <c r="D23" t="s">
-        <v>59</v>
       </c>
       <c r="F23" t="s">
         <v>25</v>
       </c>
       <c r="K23" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.25">
@@ -2157,19 +2154,19 @@
         <v>23</v>
       </c>
       <c r="B24" t="s">
+        <v>60</v>
+      </c>
+      <c r="C24" t="s">
+        <v>35</v>
+      </c>
+      <c r="D24" t="s">
         <v>61</v>
-      </c>
-      <c r="C24" t="s">
-        <v>36</v>
-      </c>
-      <c r="D24" t="s">
-        <v>62</v>
       </c>
       <c r="F24" t="s">
         <v>25</v>
       </c>
       <c r="K24" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.25">
@@ -2177,13 +2174,13 @@
         <v>24</v>
       </c>
       <c r="B25" t="s">
+        <v>63</v>
+      </c>
+      <c r="C25" t="s">
+        <v>35</v>
+      </c>
+      <c r="D25" t="s">
         <v>64</v>
-      </c>
-      <c r="C25" t="s">
-        <v>36</v>
-      </c>
-      <c r="D25" t="s">
-        <v>65</v>
       </c>
       <c r="F25" t="s">
         <v>17</v>
@@ -2194,10 +2191,10 @@
         <v>25</v>
       </c>
       <c r="B26" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C26" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="F26" t="s">
         <v>13</v>
@@ -2208,19 +2205,19 @@
         <v>26</v>
       </c>
       <c r="B27" t="s">
+        <v>66</v>
+      </c>
+      <c r="C27" t="s">
+        <v>35</v>
+      </c>
+      <c r="D27" t="s">
         <v>67</v>
       </c>
-      <c r="C27" t="s">
-        <v>36</v>
-      </c>
-      <c r="D27" t="s">
+      <c r="F27" t="s">
+        <v>52</v>
+      </c>
+      <c r="K27" t="s">
         <v>68</v>
-      </c>
-      <c r="F27" t="s">
-        <v>53</v>
-      </c>
-      <c r="K27" t="s">
-        <v>69</v>
       </c>
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.25">
@@ -2228,19 +2225,19 @@
         <v>27</v>
       </c>
       <c r="B28" t="s">
+        <v>69</v>
+      </c>
+      <c r="C28" t="s">
+        <v>35</v>
+      </c>
+      <c r="D28" t="s">
         <v>70</v>
       </c>
-      <c r="C28" t="s">
-        <v>36</v>
-      </c>
-      <c r="D28" t="s">
+      <c r="F28" t="s">
+        <v>52</v>
+      </c>
+      <c r="K28" t="s">
         <v>71</v>
-      </c>
-      <c r="F28" t="s">
-        <v>53</v>
-      </c>
-      <c r="K28" t="s">
-        <v>72</v>
       </c>
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.25">
@@ -2248,19 +2245,19 @@
         <v>28</v>
       </c>
       <c r="B29" t="s">
+        <v>72</v>
+      </c>
+      <c r="C29" t="s">
+        <v>35</v>
+      </c>
+      <c r="D29" t="s">
         <v>73</v>
       </c>
-      <c r="C29" t="s">
-        <v>36</v>
-      </c>
-      <c r="D29" t="s">
+      <c r="F29" t="s">
+        <v>52</v>
+      </c>
+      <c r="K29" t="s">
         <v>74</v>
-      </c>
-      <c r="F29" t="s">
-        <v>53</v>
-      </c>
-      <c r="K29" t="s">
-        <v>75</v>
       </c>
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.25">
@@ -2268,19 +2265,19 @@
         <v>29</v>
       </c>
       <c r="B30" t="s">
+        <v>75</v>
+      </c>
+      <c r="C30" t="s">
+        <v>35</v>
+      </c>
+      <c r="D30" t="s">
         <v>76</v>
       </c>
-      <c r="C30" t="s">
-        <v>36</v>
-      </c>
-      <c r="D30" t="s">
+      <c r="F30" t="s">
+        <v>52</v>
+      </c>
+      <c r="K30" t="s">
         <v>77</v>
-      </c>
-      <c r="F30" t="s">
-        <v>53</v>
-      </c>
-      <c r="K30" t="s">
-        <v>78</v>
       </c>
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.25">
@@ -2288,19 +2285,19 @@
         <v>30</v>
       </c>
       <c r="B31" t="s">
+        <v>78</v>
+      </c>
+      <c r="C31" t="s">
+        <v>35</v>
+      </c>
+      <c r="D31" t="s">
         <v>79</v>
       </c>
-      <c r="C31" t="s">
-        <v>36</v>
-      </c>
-      <c r="D31" t="s">
+      <c r="F31" t="s">
+        <v>52</v>
+      </c>
+      <c r="K31" t="s">
         <v>80</v>
-      </c>
-      <c r="F31" t="s">
-        <v>53</v>
-      </c>
-      <c r="K31" t="s">
-        <v>81</v>
       </c>
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.25">
@@ -2308,19 +2305,19 @@
         <v>31</v>
       </c>
       <c r="B32" t="s">
+        <v>81</v>
+      </c>
+      <c r="C32" t="s">
+        <v>35</v>
+      </c>
+      <c r="D32" t="s">
         <v>82</v>
       </c>
-      <c r="C32" t="s">
-        <v>36</v>
-      </c>
-      <c r="D32" t="s">
+      <c r="F32" t="s">
+        <v>52</v>
+      </c>
+      <c r="K32" t="s">
         <v>83</v>
-      </c>
-      <c r="F32" t="s">
-        <v>53</v>
-      </c>
-      <c r="K32" t="s">
-        <v>84</v>
       </c>
     </row>
     <row r="33" spans="1:10" x14ac:dyDescent="0.25">
@@ -2328,13 +2325,13 @@
         <v>32</v>
       </c>
       <c r="B33" t="s">
+        <v>84</v>
+      </c>
+      <c r="C33" t="s">
+        <v>35</v>
+      </c>
+      <c r="D33" t="s">
         <v>85</v>
-      </c>
-      <c r="C33" t="s">
-        <v>36</v>
-      </c>
-      <c r="D33" t="s">
-        <v>86</v>
       </c>
       <c r="F33" t="s">
         <v>17</v>
@@ -2345,10 +2342,10 @@
         <v>33</v>
       </c>
       <c r="B34" t="s">
+        <v>86</v>
+      </c>
+      <c r="C34" t="s">
         <v>87</v>
-      </c>
-      <c r="C34" t="s">
-        <v>88</v>
       </c>
       <c r="F34" t="s">
         <v>13</v>
@@ -2359,19 +2356,19 @@
         <v>34</v>
       </c>
       <c r="B35" t="s">
+        <v>88</v>
+      </c>
+      <c r="C35" t="s">
+        <v>87</v>
+      </c>
+      <c r="D35" t="s">
         <v>89</v>
       </c>
-      <c r="C35" t="s">
-        <v>88</v>
-      </c>
-      <c r="D35" t="s">
+      <c r="F35" t="s">
         <v>90</v>
       </c>
-      <c r="F35" t="s">
+      <c r="J35" t="s">
         <v>91</v>
-      </c>
-      <c r="J35" t="s">
-        <v>92</v>
       </c>
     </row>
     <row r="36" spans="1:10" x14ac:dyDescent="0.25">
@@ -2379,22 +2376,22 @@
         <v>35</v>
       </c>
       <c r="B36" t="s">
+        <v>92</v>
+      </c>
+      <c r="C36" t="s">
+        <v>87</v>
+      </c>
+      <c r="D36" t="s">
+        <v>89</v>
+      </c>
+      <c r="F36" t="s">
         <v>93</v>
       </c>
-      <c r="C36" t="s">
-        <v>88</v>
-      </c>
-      <c r="D36" t="s">
-        <v>90</v>
-      </c>
-      <c r="F36" t="s">
+      <c r="G36" t="s">
         <v>94</v>
       </c>
-      <c r="G36" t="s">
+      <c r="H36" t="s">
         <v>95</v>
-      </c>
-      <c r="H36" t="s">
-        <v>96</v>
       </c>
     </row>
     <row r="37" spans="1:10" x14ac:dyDescent="0.25">
@@ -2402,13 +2399,13 @@
         <v>36</v>
       </c>
       <c r="B37" t="s">
+        <v>96</v>
+      </c>
+      <c r="C37" t="s">
+        <v>87</v>
+      </c>
+      <c r="D37" t="s">
         <v>97</v>
-      </c>
-      <c r="C37" t="s">
-        <v>88</v>
-      </c>
-      <c r="D37" t="s">
-        <v>98</v>
       </c>
       <c r="F37" t="s">
         <v>17</v>
@@ -2419,7 +2416,7 @@
         <v>37</v>
       </c>
       <c r="B38" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="F38" t="s">
         <v>14</v>
@@ -2433,7 +2430,7 @@
         <v>38</v>
       </c>
       <c r="B39" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C39" t="s">
         <v>12</v>
@@ -2447,13 +2444,13 @@
         <v>39</v>
       </c>
       <c r="B40" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C40" t="s">
         <v>12</v>
       </c>
       <c r="D40" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="F40" t="s">
         <v>17</v>
@@ -2464,10 +2461,10 @@
         <v>40</v>
       </c>
       <c r="B41" t="s">
+        <v>102</v>
+      </c>
+      <c r="C41" t="s">
         <v>103</v>
-      </c>
-      <c r="C41" t="s">
-        <v>104</v>
       </c>
       <c r="F41" t="s">
         <v>13</v>
@@ -2478,10 +2475,10 @@
         <v>41</v>
       </c>
       <c r="B42" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="C42" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D42" t="s">
         <v>24</v>
@@ -2498,13 +2495,13 @@
         <v>42</v>
       </c>
       <c r="B43" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C43" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D43" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F43" t="s">
         <v>17</v>
@@ -2515,10 +2512,10 @@
         <v>43</v>
       </c>
       <c r="B44" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C44" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="F44" t="s">
         <v>13</v>
@@ -2529,13 +2526,13 @@
         <v>44</v>
       </c>
       <c r="B45" t="s">
+        <v>107</v>
+      </c>
+      <c r="C45" t="s">
         <v>108</v>
       </c>
-      <c r="C45" t="s">
+      <c r="D45" t="s">
         <v>109</v>
-      </c>
-      <c r="D45" t="s">
-        <v>110</v>
       </c>
       <c r="F45" t="s">
         <v>17</v>
@@ -2546,10 +2543,10 @@
         <v>45</v>
       </c>
       <c r="B46" t="s">
+        <v>110</v>
+      </c>
+      <c r="C46" t="s">
         <v>111</v>
-      </c>
-      <c r="C46" t="s">
-        <v>112</v>
       </c>
       <c r="F46" t="s">
         <v>13</v>
@@ -2560,22 +2557,22 @@
         <v>46</v>
       </c>
       <c r="B47" t="s">
+        <v>112</v>
+      </c>
+      <c r="C47" t="s">
+        <v>111</v>
+      </c>
+      <c r="D47" t="s">
         <v>113</v>
       </c>
-      <c r="C47" t="s">
-        <v>112</v>
-      </c>
-      <c r="D47" t="s">
+      <c r="F47" t="s">
+        <v>93</v>
+      </c>
+      <c r="G47" t="s">
         <v>114</v>
       </c>
-      <c r="F47" t="s">
-        <v>94</v>
-      </c>
-      <c r="G47" t="s">
+      <c r="H47" t="s">
         <v>115</v>
-      </c>
-      <c r="H47" t="s">
-        <v>116</v>
       </c>
       <c r="J47" t="b">
         <v>1</v>
@@ -2586,19 +2583,19 @@
         <v>47</v>
       </c>
       <c r="B48" t="s">
+        <v>116</v>
+      </c>
+      <c r="C48" t="s">
+        <v>111</v>
+      </c>
+      <c r="D48" t="s">
+        <v>113</v>
+      </c>
+      <c r="F48" t="s">
+        <v>90</v>
+      </c>
+      <c r="J48" t="s">
         <v>117</v>
-      </c>
-      <c r="C48" t="s">
-        <v>112</v>
-      </c>
-      <c r="D48" t="s">
-        <v>114</v>
-      </c>
-      <c r="F48" t="s">
-        <v>91</v>
-      </c>
-      <c r="J48" t="s">
-        <v>118</v>
       </c>
     </row>
     <row r="49" spans="1:11" x14ac:dyDescent="0.25">
@@ -2606,13 +2603,13 @@
         <v>48</v>
       </c>
       <c r="B49" t="s">
+        <v>118</v>
+      </c>
+      <c r="C49" t="s">
+        <v>111</v>
+      </c>
+      <c r="D49" t="s">
         <v>119</v>
-      </c>
-      <c r="C49" t="s">
-        <v>112</v>
-      </c>
-      <c r="D49" t="s">
-        <v>120</v>
       </c>
       <c r="F49" t="s">
         <v>17</v>
@@ -2623,10 +2620,10 @@
         <v>49</v>
       </c>
       <c r="B50" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="C50" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="F50" t="s">
         <v>13</v>
@@ -2637,13 +2634,13 @@
         <v>50</v>
       </c>
       <c r="B51" t="s">
+        <v>121</v>
+      </c>
+      <c r="C51" t="s">
+        <v>111</v>
+      </c>
+      <c r="D51" t="s">
         <v>122</v>
-      </c>
-      <c r="C51" t="s">
-        <v>112</v>
-      </c>
-      <c r="D51" t="s">
-        <v>123</v>
       </c>
       <c r="F51" t="s">
         <v>17</v>
@@ -2654,10 +2651,10 @@
         <v>51</v>
       </c>
       <c r="B52" t="s">
+        <v>123</v>
+      </c>
+      <c r="C52" t="s">
         <v>124</v>
-      </c>
-      <c r="C52" t="s">
-        <v>125</v>
       </c>
       <c r="F52" t="s">
         <v>13</v>
@@ -2668,19 +2665,19 @@
         <v>52</v>
       </c>
       <c r="B53" t="s">
+        <v>125</v>
+      </c>
+      <c r="C53" t="s">
+        <v>124</v>
+      </c>
+      <c r="D53" t="s">
         <v>126</v>
       </c>
-      <c r="C53" t="s">
-        <v>125</v>
-      </c>
-      <c r="D53" t="s">
+      <c r="F53" t="s">
+        <v>52</v>
+      </c>
+      <c r="K53" t="s">
         <v>127</v>
-      </c>
-      <c r="F53" t="s">
-        <v>53</v>
-      </c>
-      <c r="K53" t="s">
-        <v>128</v>
       </c>
     </row>
     <row r="54" spans="1:11" x14ac:dyDescent="0.25">
@@ -2688,19 +2685,19 @@
         <v>53</v>
       </c>
       <c r="B54" t="s">
+        <v>128</v>
+      </c>
+      <c r="C54" t="s">
+        <v>124</v>
+      </c>
+      <c r="D54" t="s">
         <v>129</v>
       </c>
-      <c r="C54" t="s">
-        <v>125</v>
-      </c>
-      <c r="D54" t="s">
+      <c r="F54" t="s">
+        <v>52</v>
+      </c>
+      <c r="K54" t="s">
         <v>130</v>
-      </c>
-      <c r="F54" t="s">
-        <v>53</v>
-      </c>
-      <c r="K54" t="s">
-        <v>131</v>
       </c>
     </row>
     <row r="55" spans="1:11" x14ac:dyDescent="0.25">
@@ -2708,19 +2705,19 @@
         <v>54</v>
       </c>
       <c r="B55" t="s">
+        <v>131</v>
+      </c>
+      <c r="C55" t="s">
+        <v>124</v>
+      </c>
+      <c r="D55" t="s">
         <v>132</v>
       </c>
-      <c r="C55" t="s">
-        <v>125</v>
-      </c>
-      <c r="D55" t="s">
+      <c r="F55" t="s">
+        <v>52</v>
+      </c>
+      <c r="K55" t="s">
         <v>133</v>
-      </c>
-      <c r="F55" t="s">
-        <v>53</v>
-      </c>
-      <c r="K55" t="s">
-        <v>134</v>
       </c>
     </row>
     <row r="56" spans="1:11" x14ac:dyDescent="0.25">
@@ -2728,19 +2725,19 @@
         <v>55</v>
       </c>
       <c r="B56" t="s">
+        <v>134</v>
+      </c>
+      <c r="C56" t="s">
+        <v>124</v>
+      </c>
+      <c r="D56" t="s">
         <v>135</v>
       </c>
-      <c r="C56" t="s">
-        <v>125</v>
-      </c>
-      <c r="D56" t="s">
+      <c r="F56" t="s">
+        <v>52</v>
+      </c>
+      <c r="K56" t="s">
         <v>136</v>
-      </c>
-      <c r="F56" t="s">
-        <v>53</v>
-      </c>
-      <c r="K56" t="s">
-        <v>137</v>
       </c>
     </row>
     <row r="57" spans="1:11" x14ac:dyDescent="0.25">
@@ -2748,19 +2745,19 @@
         <v>56</v>
       </c>
       <c r="B57" t="s">
+        <v>137</v>
+      </c>
+      <c r="C57" t="s">
+        <v>124</v>
+      </c>
+      <c r="D57" t="s">
         <v>138</v>
       </c>
-      <c r="C57" t="s">
-        <v>125</v>
-      </c>
-      <c r="D57" t="s">
+      <c r="F57" t="s">
+        <v>52</v>
+      </c>
+      <c r="K57" t="s">
         <v>139</v>
-      </c>
-      <c r="F57" t="s">
-        <v>53</v>
-      </c>
-      <c r="K57" t="s">
-        <v>140</v>
       </c>
     </row>
     <row r="58" spans="1:11" x14ac:dyDescent="0.25">
@@ -2768,13 +2765,13 @@
         <v>57</v>
       </c>
       <c r="B58" t="s">
+        <v>140</v>
+      </c>
+      <c r="C58" t="s">
+        <v>124</v>
+      </c>
+      <c r="D58" t="s">
         <v>141</v>
-      </c>
-      <c r="C58" t="s">
-        <v>125</v>
-      </c>
-      <c r="D58" t="s">
-        <v>142</v>
       </c>
       <c r="F58" t="s">
         <v>17</v>
@@ -2785,10 +2782,10 @@
         <v>58</v>
       </c>
       <c r="B59" t="s">
+        <v>142</v>
+      </c>
+      <c r="C59" t="s">
         <v>143</v>
-      </c>
-      <c r="C59" t="s">
-        <v>144</v>
       </c>
       <c r="F59" t="s">
         <v>13</v>
@@ -2799,13 +2796,13 @@
         <v>59</v>
       </c>
       <c r="B60" t="s">
+        <v>144</v>
+      </c>
+      <c r="C60" t="s">
+        <v>143</v>
+      </c>
+      <c r="D60" t="s">
         <v>145</v>
-      </c>
-      <c r="C60" t="s">
-        <v>144</v>
-      </c>
-      <c r="D60" t="s">
-        <v>146</v>
       </c>
       <c r="F60" t="s">
         <v>17</v>
@@ -2816,7 +2813,7 @@
         <v>60</v>
       </c>
       <c r="B61" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="F61" t="s">
         <v>14</v>
@@ -2830,10 +2827,10 @@
         <v>61</v>
       </c>
       <c r="B62" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="C62" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="F62" t="s">
         <v>13</v>
@@ -2844,13 +2841,13 @@
         <v>62</v>
       </c>
       <c r="B63" t="s">
+        <v>148</v>
+      </c>
+      <c r="C63" t="s">
+        <v>111</v>
+      </c>
+      <c r="D63" t="s">
         <v>149</v>
-      </c>
-      <c r="C63" t="s">
-        <v>112</v>
-      </c>
-      <c r="D63" t="s">
-        <v>150</v>
       </c>
       <c r="F63" t="s">
         <v>17</v>
@@ -2861,10 +2858,10 @@
         <v>63</v>
       </c>
       <c r="B64" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C64" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="F64" t="s">
         <v>13</v>
@@ -2875,7 +2872,7 @@
         <v>64</v>
       </c>
       <c r="B65" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="F65" t="s">
         <v>14</v>
@@ -2889,13 +2886,13 @@
         <v>65</v>
       </c>
       <c r="B66" t="s">
+        <v>152</v>
+      </c>
+      <c r="C66" t="s">
+        <v>111</v>
+      </c>
+      <c r="D66" t="s">
         <v>153</v>
-      </c>
-      <c r="C66" t="s">
-        <v>112</v>
-      </c>
-      <c r="D66" t="s">
-        <v>154</v>
       </c>
       <c r="F66" t="s">
         <v>17</v>
@@ -2906,10 +2903,10 @@
         <v>66</v>
       </c>
       <c r="B67" t="s">
+        <v>154</v>
+      </c>
+      <c r="C67" t="s">
         <v>155</v>
-      </c>
-      <c r="C67" t="s">
-        <v>156</v>
       </c>
       <c r="F67" t="s">
         <v>13</v>
@@ -2920,19 +2917,19 @@
         <v>67</v>
       </c>
       <c r="B68" t="s">
+        <v>156</v>
+      </c>
+      <c r="C68" t="s">
+        <v>155</v>
+      </c>
+      <c r="D68" t="s">
         <v>157</v>
       </c>
-      <c r="C68" t="s">
-        <v>156</v>
-      </c>
-      <c r="D68" t="s">
+      <c r="F68" t="s">
+        <v>52</v>
+      </c>
+      <c r="K68" t="s">
         <v>158</v>
-      </c>
-      <c r="F68" t="s">
-        <v>53</v>
-      </c>
-      <c r="K68" t="s">
-        <v>159</v>
       </c>
     </row>
     <row r="69" spans="1:11" x14ac:dyDescent="0.25">
@@ -2940,13 +2937,13 @@
         <v>68</v>
       </c>
       <c r="B69" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="C69" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="D69" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="F69" t="s">
         <v>17</v>
@@ -2957,10 +2954,10 @@
         <v>69</v>
       </c>
       <c r="B70" t="s">
+        <v>160</v>
+      </c>
+      <c r="C70" t="s">
         <v>161</v>
-      </c>
-      <c r="C70" t="s">
-        <v>162</v>
       </c>
       <c r="F70" t="s">
         <v>13</v>
@@ -2971,19 +2968,19 @@
         <v>70</v>
       </c>
       <c r="B71" t="s">
+        <v>162</v>
+      </c>
+      <c r="C71" t="s">
+        <v>161</v>
+      </c>
+      <c r="D71" t="s">
         <v>163</v>
       </c>
-      <c r="C71" t="s">
-        <v>162</v>
-      </c>
-      <c r="D71" t="s">
+      <c r="F71" t="s">
+        <v>52</v>
+      </c>
+      <c r="K71" t="s">
         <v>164</v>
-      </c>
-      <c r="F71" t="s">
-        <v>53</v>
-      </c>
-      <c r="K71" t="s">
-        <v>165</v>
       </c>
     </row>
     <row r="72" spans="1:11" x14ac:dyDescent="0.25">
@@ -2991,19 +2988,19 @@
         <v>71</v>
       </c>
       <c r="B72" t="s">
+        <v>165</v>
+      </c>
+      <c r="C72" t="s">
+        <v>161</v>
+      </c>
+      <c r="D72" t="s">
         <v>166</v>
       </c>
-      <c r="C72" t="s">
-        <v>162</v>
-      </c>
-      <c r="D72" t="s">
+      <c r="F72" t="s">
+        <v>52</v>
+      </c>
+      <c r="K72" t="s">
         <v>167</v>
-      </c>
-      <c r="F72" t="s">
-        <v>53</v>
-      </c>
-      <c r="K72" t="s">
-        <v>168</v>
       </c>
     </row>
     <row r="73" spans="1:11" x14ac:dyDescent="0.25">
@@ -3011,19 +3008,19 @@
         <v>72</v>
       </c>
       <c r="B73" t="s">
+        <v>168</v>
+      </c>
+      <c r="C73" t="s">
+        <v>161</v>
+      </c>
+      <c r="D73" t="s">
         <v>169</v>
       </c>
-      <c r="C73" t="s">
-        <v>162</v>
-      </c>
-      <c r="D73" t="s">
+      <c r="F73" t="s">
+        <v>52</v>
+      </c>
+      <c r="K73" t="s">
         <v>170</v>
-      </c>
-      <c r="F73" t="s">
-        <v>53</v>
-      </c>
-      <c r="K73" t="s">
-        <v>171</v>
       </c>
     </row>
     <row r="74" spans="1:11" x14ac:dyDescent="0.25">
@@ -3031,19 +3028,19 @@
         <v>73</v>
       </c>
       <c r="B74" t="s">
+        <v>171</v>
+      </c>
+      <c r="C74" t="s">
+        <v>161</v>
+      </c>
+      <c r="D74" t="s">
         <v>172</v>
       </c>
-      <c r="C74" t="s">
-        <v>162</v>
-      </c>
-      <c r="D74" t="s">
+      <c r="F74" t="s">
+        <v>52</v>
+      </c>
+      <c r="K74" t="s">
         <v>173</v>
-      </c>
-      <c r="F74" t="s">
-        <v>53</v>
-      </c>
-      <c r="K74" t="s">
-        <v>174</v>
       </c>
     </row>
     <row r="75" spans="1:11" x14ac:dyDescent="0.25">
@@ -3051,19 +3048,19 @@
         <v>74</v>
       </c>
       <c r="B75" t="s">
+        <v>174</v>
+      </c>
+      <c r="C75" t="s">
+        <v>161</v>
+      </c>
+      <c r="D75" t="s">
         <v>175</v>
       </c>
-      <c r="C75" t="s">
-        <v>162</v>
-      </c>
-      <c r="D75" t="s">
+      <c r="F75" t="s">
+        <v>52</v>
+      </c>
+      <c r="K75" t="s">
         <v>176</v>
-      </c>
-      <c r="F75" t="s">
-        <v>53</v>
-      </c>
-      <c r="K75" t="s">
-        <v>177</v>
       </c>
     </row>
     <row r="76" spans="1:11" x14ac:dyDescent="0.25">
@@ -3071,19 +3068,19 @@
         <v>75</v>
       </c>
       <c r="B76" t="s">
+        <v>177</v>
+      </c>
+      <c r="C76" t="s">
+        <v>161</v>
+      </c>
+      <c r="D76" t="s">
         <v>178</v>
       </c>
-      <c r="C76" t="s">
-        <v>162</v>
-      </c>
-      <c r="D76" t="s">
+      <c r="F76" t="s">
+        <v>52</v>
+      </c>
+      <c r="K76" t="s">
         <v>179</v>
-      </c>
-      <c r="F76" t="s">
-        <v>53</v>
-      </c>
-      <c r="K76" t="s">
-        <v>180</v>
       </c>
     </row>
     <row r="77" spans="1:11" x14ac:dyDescent="0.25">
@@ -3091,13 +3088,13 @@
         <v>76</v>
       </c>
       <c r="B77" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="C77" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="D77" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="F77" t="s">
         <v>17</v>
@@ -3108,10 +3105,10 @@
         <v>77</v>
       </c>
       <c r="B78" t="s">
+        <v>181</v>
+      </c>
+      <c r="C78" t="s">
         <v>182</v>
-      </c>
-      <c r="C78" t="s">
-        <v>183</v>
       </c>
       <c r="F78" t="s">
         <v>13</v>
@@ -3122,19 +3119,19 @@
         <v>78</v>
       </c>
       <c r="B79" t="s">
+        <v>183</v>
+      </c>
+      <c r="C79" t="s">
+        <v>182</v>
+      </c>
+      <c r="D79" t="s">
         <v>184</v>
-      </c>
-      <c r="C79" t="s">
-        <v>183</v>
-      </c>
-      <c r="D79" t="s">
-        <v>185</v>
       </c>
       <c r="F79" t="s">
         <v>25</v>
       </c>
       <c r="K79" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
     <row r="80" spans="1:11" x14ac:dyDescent="0.25">
@@ -3142,19 +3139,19 @@
         <v>79</v>
       </c>
       <c r="B80" t="s">
+        <v>186</v>
+      </c>
+      <c r="C80" t="s">
+        <v>182</v>
+      </c>
+      <c r="D80" t="s">
         <v>187</v>
       </c>
-      <c r="C80" t="s">
-        <v>183</v>
-      </c>
-      <c r="D80" t="s">
+      <c r="F80" t="s">
+        <v>52</v>
+      </c>
+      <c r="K80" t="s">
         <v>188</v>
-      </c>
-      <c r="F80" t="s">
-        <v>53</v>
-      </c>
-      <c r="K80" t="s">
-        <v>189</v>
       </c>
     </row>
     <row r="81" spans="1:11" x14ac:dyDescent="0.25">
@@ -3162,13 +3159,13 @@
         <v>80</v>
       </c>
       <c r="B81" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C81" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="D81" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="F81" t="s">
         <v>17</v>
@@ -3179,10 +3176,10 @@
         <v>81</v>
       </c>
       <c r="B82" t="s">
+        <v>190</v>
+      </c>
+      <c r="C82" t="s">
         <v>191</v>
-      </c>
-      <c r="C82" t="s">
-        <v>192</v>
       </c>
       <c r="F82" t="s">
         <v>13</v>
@@ -3193,19 +3190,19 @@
         <v>82</v>
       </c>
       <c r="B83" t="s">
+        <v>192</v>
+      </c>
+      <c r="C83" t="s">
+        <v>191</v>
+      </c>
+      <c r="D83" t="s">
         <v>193</v>
       </c>
-      <c r="C83" t="s">
-        <v>192</v>
-      </c>
-      <c r="D83" t="s">
-        <v>194</v>
-      </c>
       <c r="F83" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="G83" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="H83" t="b">
         <v>1</v>
@@ -3216,7 +3213,7 @@
         <v>83</v>
       </c>
       <c r="B84" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="F84" t="s">
         <v>14</v>
@@ -3230,13 +3227,13 @@
         <v>84</v>
       </c>
       <c r="B85" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="C85" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="D85" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="F85" t="s">
         <v>17</v>
@@ -3247,13 +3244,13 @@
         <v>85</v>
       </c>
       <c r="B86" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="C86" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="D86" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="F86" t="s">
         <v>17</v>
@@ -3264,10 +3261,10 @@
         <v>86</v>
       </c>
       <c r="B87" t="s">
+        <v>197</v>
+      </c>
+      <c r="C87" t="s">
         <v>198</v>
-      </c>
-      <c r="C87" t="s">
-        <v>199</v>
       </c>
       <c r="F87" t="s">
         <v>13</v>
@@ -3278,13 +3275,13 @@
         <v>87</v>
       </c>
       <c r="B88" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="C88" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="D88" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="F88" t="s">
         <v>17</v>
@@ -3295,10 +3292,10 @@
         <v>88</v>
       </c>
       <c r="B89" t="s">
+        <v>200</v>
+      </c>
+      <c r="C89" t="s">
         <v>201</v>
-      </c>
-      <c r="C89" t="s">
-        <v>202</v>
       </c>
       <c r="F89" t="s">
         <v>13</v>
@@ -3309,19 +3306,19 @@
         <v>89</v>
       </c>
       <c r="B90" t="s">
+        <v>202</v>
+      </c>
+      <c r="C90" t="s">
+        <v>201</v>
+      </c>
+      <c r="D90" t="s">
+        <v>175</v>
+      </c>
+      <c r="F90" t="s">
+        <v>52</v>
+      </c>
+      <c r="K90" t="s">
         <v>203</v>
-      </c>
-      <c r="C90" t="s">
-        <v>202</v>
-      </c>
-      <c r="D90" t="s">
-        <v>176</v>
-      </c>
-      <c r="F90" t="s">
-        <v>53</v>
-      </c>
-      <c r="K90" t="s">
-        <v>204</v>
       </c>
     </row>
     <row r="91" spans="1:11" x14ac:dyDescent="0.25">
@@ -3329,19 +3326,19 @@
         <v>90</v>
       </c>
       <c r="B91" t="s">
+        <v>204</v>
+      </c>
+      <c r="C91" t="s">
+        <v>201</v>
+      </c>
+      <c r="D91" t="s">
+        <v>178</v>
+      </c>
+      <c r="F91" t="s">
+        <v>52</v>
+      </c>
+      <c r="K91" t="s">
         <v>205</v>
-      </c>
-      <c r="C91" t="s">
-        <v>202</v>
-      </c>
-      <c r="D91" t="s">
-        <v>179</v>
-      </c>
-      <c r="F91" t="s">
-        <v>53</v>
-      </c>
-      <c r="K91" t="s">
-        <v>206</v>
       </c>
     </row>
     <row r="92" spans="1:11" x14ac:dyDescent="0.25">
@@ -3349,13 +3346,13 @@
         <v>91</v>
       </c>
       <c r="B92" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="C92" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="D92" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="F92" t="s">
         <v>17</v>
@@ -3366,10 +3363,10 @@
         <v>92</v>
       </c>
       <c r="B93" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="C93" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="F93" t="s">
         <v>13</v>
@@ -3380,19 +3377,19 @@
         <v>93</v>
       </c>
       <c r="B94" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="C94" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="D94" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="F94" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="G94" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="H94" t="b">
         <v>1</v>
@@ -3403,7 +3400,7 @@
         <v>94</v>
       </c>
       <c r="B95" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="F95" t="s">
         <v>14</v>
@@ -3417,13 +3414,13 @@
         <v>95</v>
       </c>
       <c r="B96" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="C96" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="D96" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="F96" t="s">
         <v>17</v>
@@ -3434,13 +3431,13 @@
         <v>96</v>
       </c>
       <c r="B97" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="C97" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="D97" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="F97" t="s">
         <v>17</v>
@@ -3451,10 +3448,10 @@
         <v>97</v>
       </c>
       <c r="B98" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="C98" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="F98" t="s">
         <v>13</v>
@@ -3465,13 +3462,13 @@
         <v>98</v>
       </c>
       <c r="B99" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="C99" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="D99" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="F99" t="s">
         <v>17</v>
@@ -3482,10 +3479,10 @@
         <v>99</v>
       </c>
       <c r="B100" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="C100" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="F100" t="s">
         <v>13</v>
@@ -3496,19 +3493,19 @@
         <v>100</v>
       </c>
       <c r="B101" t="s">
+        <v>215</v>
+      </c>
+      <c r="C101" t="s">
+        <v>201</v>
+      </c>
+      <c r="D101" t="s">
+        <v>175</v>
+      </c>
+      <c r="F101" t="s">
+        <v>52</v>
+      </c>
+      <c r="K101" t="s">
         <v>216</v>
-      </c>
-      <c r="C101" t="s">
-        <v>202</v>
-      </c>
-      <c r="D101" t="s">
-        <v>176</v>
-      </c>
-      <c r="F101" t="s">
-        <v>53</v>
-      </c>
-      <c r="K101" t="s">
-        <v>217</v>
       </c>
     </row>
     <row r="102" spans="1:11" x14ac:dyDescent="0.25">
@@ -3516,19 +3513,19 @@
         <v>101</v>
       </c>
       <c r="B102" t="s">
+        <v>217</v>
+      </c>
+      <c r="C102" t="s">
+        <v>201</v>
+      </c>
+      <c r="D102" t="s">
+        <v>178</v>
+      </c>
+      <c r="F102" t="s">
+        <v>52</v>
+      </c>
+      <c r="K102" t="s">
         <v>218</v>
-      </c>
-      <c r="C102" t="s">
-        <v>202</v>
-      </c>
-      <c r="D102" t="s">
-        <v>179</v>
-      </c>
-      <c r="F102" t="s">
-        <v>53</v>
-      </c>
-      <c r="K102" t="s">
-        <v>219</v>
       </c>
     </row>
     <row r="103" spans="1:11" x14ac:dyDescent="0.25">
@@ -3536,13 +3533,13 @@
         <v>102</v>
       </c>
       <c r="B103" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="C103" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="D103" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="F103" t="s">
         <v>17</v>
@@ -3553,10 +3550,10 @@
         <v>103</v>
       </c>
       <c r="B104" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="C104" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="F104" t="s">
         <v>13</v>
@@ -3567,19 +3564,19 @@
         <v>104</v>
       </c>
       <c r="B105" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="C105" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="D105" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="F105" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="G105" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="H105" t="b">
         <v>1</v>
@@ -3590,7 +3587,7 @@
         <v>105</v>
       </c>
       <c r="B106" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="F106" t="s">
         <v>14</v>
@@ -3604,10 +3601,10 @@
         <v>106</v>
       </c>
       <c r="B107" t="s">
+        <v>223</v>
+      </c>
+      <c r="C107" t="s">
         <v>224</v>
-      </c>
-      <c r="C107" t="s">
-        <v>225</v>
       </c>
       <c r="F107" t="s">
         <v>13</v>
@@ -3618,19 +3615,19 @@
         <v>107</v>
       </c>
       <c r="B108" t="s">
+        <v>225</v>
+      </c>
+      <c r="C108" t="s">
+        <v>224</v>
+      </c>
+      <c r="D108" t="s">
         <v>226</v>
       </c>
-      <c r="C108" t="s">
-        <v>225</v>
-      </c>
-      <c r="D108" t="s">
+      <c r="F108" t="s">
+        <v>52</v>
+      </c>
+      <c r="K108" t="s">
         <v>227</v>
-      </c>
-      <c r="F108" t="s">
-        <v>53</v>
-      </c>
-      <c r="K108" t="s">
-        <v>228</v>
       </c>
     </row>
     <row r="109" spans="1:11" x14ac:dyDescent="0.25">
@@ -3638,19 +3635,19 @@
         <v>108</v>
       </c>
       <c r="B109" t="s">
+        <v>228</v>
+      </c>
+      <c r="C109" t="s">
+        <v>224</v>
+      </c>
+      <c r="D109" t="s">
         <v>229</v>
       </c>
-      <c r="C109" t="s">
-        <v>225</v>
-      </c>
-      <c r="D109" t="s">
+      <c r="F109" t="s">
+        <v>52</v>
+      </c>
+      <c r="K109" t="s">
         <v>230</v>
-      </c>
-      <c r="F109" t="s">
-        <v>53</v>
-      </c>
-      <c r="K109" t="s">
-        <v>231</v>
       </c>
     </row>
     <row r="110" spans="1:11" x14ac:dyDescent="0.25">
@@ -3658,13 +3655,13 @@
         <v>109</v>
       </c>
       <c r="B110" t="s">
+        <v>231</v>
+      </c>
+      <c r="C110" t="s">
+        <v>224</v>
+      </c>
+      <c r="D110" t="s">
         <v>232</v>
-      </c>
-      <c r="C110" t="s">
-        <v>225</v>
-      </c>
-      <c r="D110" t="s">
-        <v>233</v>
       </c>
       <c r="F110" t="s">
         <v>17</v>
@@ -3675,10 +3672,10 @@
         <v>110</v>
       </c>
       <c r="B111" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="C111" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="F111" t="s">
         <v>13</v>
@@ -3689,13 +3686,13 @@
         <v>111</v>
       </c>
       <c r="B112" t="s">
+        <v>234</v>
+      </c>
+      <c r="C112" t="s">
+        <v>224</v>
+      </c>
+      <c r="D112" t="s">
         <v>235</v>
-      </c>
-      <c r="C112" t="s">
-        <v>225</v>
-      </c>
-      <c r="D112" t="s">
-        <v>236</v>
       </c>
       <c r="F112" t="s">
         <v>17</v>
@@ -3706,13 +3703,13 @@
         <v>112</v>
       </c>
       <c r="B113" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="C113" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="D113" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="F113" t="s">
         <v>17</v>
@@ -3723,10 +3720,10 @@
         <v>113</v>
       </c>
       <c r="B114" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="C114" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="F114" t="s">
         <v>13</v>
@@ -3737,19 +3734,19 @@
         <v>114</v>
       </c>
       <c r="B115" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="C115" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="D115" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="F115" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="G115" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="H115" t="b">
         <v>1</v>
@@ -3760,7 +3757,7 @@
         <v>115</v>
       </c>
       <c r="B116" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="F116" t="s">
         <v>14</v>
@@ -3774,10 +3771,10 @@
         <v>116</v>
       </c>
       <c r="B117" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="C117" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="F117" t="s">
         <v>13</v>
@@ -3788,19 +3785,19 @@
         <v>117</v>
       </c>
       <c r="B118" t="s">
+        <v>241</v>
+      </c>
+      <c r="C118" t="s">
+        <v>224</v>
+      </c>
+      <c r="D118" t="s">
+        <v>226</v>
+      </c>
+      <c r="F118" t="s">
+        <v>52</v>
+      </c>
+      <c r="K118" t="s">
         <v>242</v>
-      </c>
-      <c r="C118" t="s">
-        <v>225</v>
-      </c>
-      <c r="D118" t="s">
-        <v>227</v>
-      </c>
-      <c r="F118" t="s">
-        <v>53</v>
-      </c>
-      <c r="K118" t="s">
-        <v>243</v>
       </c>
     </row>
     <row r="119" spans="1:11" x14ac:dyDescent="0.25">
@@ -3808,19 +3805,19 @@
         <v>118</v>
       </c>
       <c r="B119" t="s">
+        <v>243</v>
+      </c>
+      <c r="C119" t="s">
+        <v>224</v>
+      </c>
+      <c r="D119" t="s">
+        <v>229</v>
+      </c>
+      <c r="F119" t="s">
+        <v>52</v>
+      </c>
+      <c r="K119" t="s">
         <v>244</v>
-      </c>
-      <c r="C119" t="s">
-        <v>225</v>
-      </c>
-      <c r="D119" t="s">
-        <v>230</v>
-      </c>
-      <c r="F119" t="s">
-        <v>53</v>
-      </c>
-      <c r="K119" t="s">
-        <v>245</v>
       </c>
     </row>
     <row r="120" spans="1:11" x14ac:dyDescent="0.25">
@@ -3828,13 +3825,13 @@
         <v>119</v>
       </c>
       <c r="B120" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="C120" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="D120" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="F120" t="s">
         <v>17</v>
@@ -3845,10 +3842,10 @@
         <v>120</v>
       </c>
       <c r="B121" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="C121" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="F121" t="s">
         <v>13</v>
@@ -3859,13 +3856,13 @@
         <v>121</v>
       </c>
       <c r="B122" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="C122" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="D122" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="F122" t="s">
         <v>17</v>
@@ -3876,13 +3873,13 @@
         <v>122</v>
       </c>
       <c r="B123" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="C123" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="D123" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="F123" t="s">
         <v>17</v>
@@ -3893,10 +3890,10 @@
         <v>123</v>
       </c>
       <c r="B124" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="C124" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="F124" t="s">
         <v>13</v>
@@ -3907,19 +3904,19 @@
         <v>124</v>
       </c>
       <c r="B125" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="C125" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="D125" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="F125" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="G125" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="H125" t="b">
         <v>1</v>
@@ -3930,7 +3927,7 @@
         <v>125</v>
       </c>
       <c r="B126" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="F126" t="s">
         <v>14</v>
@@ -3944,13 +3941,13 @@
         <v>126</v>
       </c>
       <c r="B127" t="s">
+        <v>252</v>
+      </c>
+      <c r="C127" t="s">
         <v>253</v>
       </c>
-      <c r="C127" t="s">
+      <c r="D127" t="s">
         <v>254</v>
-      </c>
-      <c r="D127" t="s">
-        <v>255</v>
       </c>
       <c r="F127" t="s">
         <v>17</v>
@@ -3961,10 +3958,10 @@
         <v>127</v>
       </c>
       <c r="B128" t="s">
+        <v>255</v>
+      </c>
+      <c r="C128" t="s">
         <v>256</v>
-      </c>
-      <c r="C128" t="s">
-        <v>257</v>
       </c>
       <c r="F128" t="s">
         <v>13</v>
@@ -3975,13 +3972,13 @@
         <v>128</v>
       </c>
       <c r="B129" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="C129" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="D129" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="F129" t="s">
         <v>17</v>
@@ -3992,10 +3989,10 @@
         <v>129</v>
       </c>
       <c r="B130" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="C130" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="F130" t="s">
         <v>13</v>
@@ -4006,13 +4003,13 @@
         <v>130</v>
       </c>
       <c r="B131" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="C131" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="D131" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="F131" t="s">
         <v>17</v>
@@ -4023,10 +4020,10 @@
         <v>131</v>
       </c>
       <c r="B132" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="C132" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="F132" t="s">
         <v>13</v>
@@ -4037,13 +4034,13 @@
         <v>132</v>
       </c>
       <c r="B133" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="C133" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="D133" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="F133" t="s">
         <v>17</v>
@@ -4054,10 +4051,10 @@
         <v>133</v>
       </c>
       <c r="B134" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="C134" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="F134" t="s">
         <v>13</v>
@@ -4068,19 +4065,19 @@
         <v>134</v>
       </c>
       <c r="B135" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="C135" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="D135" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="F135" t="s">
         <v>25</v>
       </c>
       <c r="K135" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
     </row>
     <row r="136" spans="1:11" x14ac:dyDescent="0.25">
@@ -4088,19 +4085,19 @@
         <v>135</v>
       </c>
       <c r="B136" t="s">
+        <v>265</v>
+      </c>
+      <c r="C136" t="s">
+        <v>182</v>
+      </c>
+      <c r="D136" t="s">
+        <v>187</v>
+      </c>
+      <c r="F136" t="s">
+        <v>52</v>
+      </c>
+      <c r="K136" t="s">
         <v>266</v>
-      </c>
-      <c r="C136" t="s">
-        <v>183</v>
-      </c>
-      <c r="D136" t="s">
-        <v>188</v>
-      </c>
-      <c r="F136" t="s">
-        <v>53</v>
-      </c>
-      <c r="K136" t="s">
-        <v>267</v>
       </c>
     </row>
     <row r="137" spans="1:11" x14ac:dyDescent="0.25">
@@ -4108,13 +4105,13 @@
         <v>136</v>
       </c>
       <c r="B137" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="C137" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="D137" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="F137" t="s">
         <v>17</v>
@@ -4125,10 +4122,10 @@
         <v>137</v>
       </c>
       <c r="B138" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="C138" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="F138" t="s">
         <v>13</v>
@@ -4139,19 +4136,19 @@
         <v>138</v>
       </c>
       <c r="B139" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="C139" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="D139" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="F139" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="G139" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="H139" t="b">
         <v>1</v>
@@ -4162,7 +4159,7 @@
         <v>139</v>
       </c>
       <c r="B140" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="F140" t="s">
         <v>14</v>
@@ -4176,10 +4173,10 @@
         <v>140</v>
       </c>
       <c r="B141" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="C141" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="F141" t="s">
         <v>13</v>
@@ -4190,13 +4187,13 @@
         <v>141</v>
       </c>
       <c r="B142" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="C142" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="D142" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="F142" t="s">
         <v>17</v>
@@ -4207,10 +4204,10 @@
         <v>142</v>
       </c>
       <c r="B143" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="C143" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="F143" t="s">
         <v>13</v>
@@ -4221,19 +4218,19 @@
         <v>143</v>
       </c>
       <c r="B144" t="s">
+        <v>274</v>
+      </c>
+      <c r="C144" t="s">
+        <v>191</v>
+      </c>
+      <c r="D144" t="s">
         <v>275</v>
       </c>
-      <c r="C144" t="s">
-        <v>192</v>
-      </c>
-      <c r="D144" t="s">
-        <v>276</v>
-      </c>
       <c r="F144" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="G144" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="H144" t="b">
         <v>1</v>
@@ -4244,7 +4241,7 @@
         <v>144</v>
       </c>
       <c r="B145" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="F145" t="s">
         <v>14</v>
@@ -4258,13 +4255,13 @@
         <v>145</v>
       </c>
       <c r="B146" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="C146" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="D146" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="F146" t="s">
         <v>17</v>
@@ -4275,13 +4272,13 @@
         <v>146</v>
       </c>
       <c r="B147" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="C147" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="D147" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="F147" t="s">
         <v>17</v>
@@ -4292,10 +4289,10 @@
         <v>147</v>
       </c>
       <c r="B148" t="s">
+        <v>279</v>
+      </c>
+      <c r="C148" t="s">
         <v>280</v>
-      </c>
-      <c r="C148" t="s">
-        <v>281</v>
       </c>
       <c r="F148" t="s">
         <v>13</v>
@@ -4306,13 +4303,13 @@
         <v>148</v>
       </c>
       <c r="B149" t="s">
+        <v>281</v>
+      </c>
+      <c r="C149" t="s">
+        <v>280</v>
+      </c>
+      <c r="D149" t="s">
         <v>282</v>
-      </c>
-      <c r="C149" t="s">
-        <v>281</v>
-      </c>
-      <c r="D149" t="s">
-        <v>283</v>
       </c>
       <c r="F149" t="s">
         <v>17</v>
@@ -4323,19 +4320,19 @@
         <v>149</v>
       </c>
       <c r="B150" t="s">
+        <v>283</v>
+      </c>
+      <c r="C150" t="s">
+        <v>280</v>
+      </c>
+      <c r="D150" t="s">
         <v>284</v>
-      </c>
-      <c r="C150" t="s">
-        <v>281</v>
-      </c>
-      <c r="D150" t="s">
-        <v>285</v>
       </c>
       <c r="F150" t="s">
         <v>25</v>
       </c>
       <c r="K150" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="151" spans="1:11" x14ac:dyDescent="0.25">
@@ -4343,19 +4340,19 @@
         <v>150</v>
       </c>
       <c r="B151" t="s">
+        <v>286</v>
+      </c>
+      <c r="C151" t="s">
+        <v>280</v>
+      </c>
+      <c r="D151" t="s">
         <v>287</v>
       </c>
-      <c r="C151" t="s">
-        <v>281</v>
-      </c>
-      <c r="D151" t="s">
+      <c r="F151" t="s">
+        <v>52</v>
+      </c>
+      <c r="K151" t="s">
         <v>288</v>
-      </c>
-      <c r="F151" t="s">
-        <v>53</v>
-      </c>
-      <c r="K151" t="s">
-        <v>289</v>
       </c>
     </row>
     <row r="152" spans="1:11" x14ac:dyDescent="0.25">
@@ -4363,19 +4360,19 @@
         <v>151</v>
       </c>
       <c r="B152" t="s">
+        <v>289</v>
+      </c>
+      <c r="C152" t="s">
+        <v>280</v>
+      </c>
+      <c r="D152" t="s">
         <v>290</v>
-      </c>
-      <c r="C152" t="s">
-        <v>281</v>
-      </c>
-      <c r="D152" t="s">
-        <v>291</v>
       </c>
       <c r="F152" t="s">
         <v>25</v>
       </c>
       <c r="K152" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
     </row>
     <row r="153" spans="1:11" x14ac:dyDescent="0.25">
@@ -4383,13 +4380,13 @@
         <v>152</v>
       </c>
       <c r="B153" t="s">
+        <v>292</v>
+      </c>
+      <c r="C153" t="s">
+        <v>280</v>
+      </c>
+      <c r="D153" t="s">
         <v>293</v>
-      </c>
-      <c r="C153" t="s">
-        <v>281</v>
-      </c>
-      <c r="D153" t="s">
-        <v>294</v>
       </c>
       <c r="F153" t="s">
         <v>17</v>
@@ -4400,10 +4397,10 @@
         <v>153</v>
       </c>
       <c r="B154" t="s">
+        <v>294</v>
+      </c>
+      <c r="C154" t="s">
         <v>295</v>
-      </c>
-      <c r="C154" t="s">
-        <v>296</v>
       </c>
       <c r="F154" t="s">
         <v>13</v>
@@ -4414,13 +4411,13 @@
         <v>154</v>
       </c>
       <c r="B155" t="s">
+        <v>296</v>
+      </c>
+      <c r="C155" t="s">
+        <v>295</v>
+      </c>
+      <c r="D155" t="s">
         <v>297</v>
-      </c>
-      <c r="C155" t="s">
-        <v>296</v>
-      </c>
-      <c r="D155" t="s">
-        <v>298</v>
       </c>
       <c r="F155" t="s">
         <v>17</v>
@@ -4431,10 +4428,10 @@
         <v>155</v>
       </c>
       <c r="B156" t="s">
+        <v>298</v>
+      </c>
+      <c r="C156" t="s">
         <v>299</v>
-      </c>
-      <c r="C156" t="s">
-        <v>300</v>
       </c>
       <c r="F156" t="s">
         <v>13</v>
@@ -4445,13 +4442,13 @@
         <v>156</v>
       </c>
       <c r="B157" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="C157" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="D157" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="F157" t="s">
         <v>17</v>
@@ -4462,13 +4459,13 @@
         <v>157</v>
       </c>
       <c r="B158" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="C158" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="D158" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="F158" t="s">
         <v>17</v>
@@ -4479,10 +4476,10 @@
         <v>158</v>
       </c>
       <c r="B159" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="C159" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="F159" t="s">
         <v>13</v>
@@ -4493,19 +4490,19 @@
         <v>159</v>
       </c>
       <c r="B160" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="C160" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="D160" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="F160" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="G160" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="H160" t="b">
         <v>1</v>
@@ -4516,7 +4513,7 @@
         <v>160</v>
       </c>
       <c r="B161" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="F161" t="s">
         <v>14</v>
@@ -4530,13 +4527,13 @@
         <v>161</v>
       </c>
       <c r="B162" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="C162" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="D162" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="F162" t="s">
         <v>17</v>
@@ -4547,10 +4544,10 @@
         <v>162</v>
       </c>
       <c r="B163" t="s">
+        <v>306</v>
+      </c>
+      <c r="C163" t="s">
         <v>307</v>
-      </c>
-      <c r="C163" t="s">
-        <v>308</v>
       </c>
       <c r="F163" t="s">
         <v>13</v>
@@ -4561,13 +4558,13 @@
         <v>163</v>
       </c>
       <c r="B164" t="s">
+        <v>308</v>
+      </c>
+      <c r="C164" t="s">
+        <v>307</v>
+      </c>
+      <c r="D164" t="s">
         <v>309</v>
-      </c>
-      <c r="C164" t="s">
-        <v>308</v>
-      </c>
-      <c r="D164" t="s">
-        <v>310</v>
       </c>
       <c r="F164" t="s">
         <v>17</v>
@@ -4578,13 +4575,13 @@
         <v>164</v>
       </c>
       <c r="B165" t="s">
+        <v>310</v>
+      </c>
+      <c r="C165" t="s">
+        <v>307</v>
+      </c>
+      <c r="D165" t="s">
         <v>311</v>
-      </c>
-      <c r="C165" t="s">
-        <v>308</v>
-      </c>
-      <c r="D165" t="s">
-        <v>312</v>
       </c>
       <c r="F165" t="s">
         <v>17</v>
@@ -4595,10 +4592,10 @@
         <v>165</v>
       </c>
       <c r="B166" t="s">
+        <v>312</v>
+      </c>
+      <c r="C166" t="s">
         <v>313</v>
-      </c>
-      <c r="C166" t="s">
-        <v>314</v>
       </c>
       <c r="F166" t="s">
         <v>13</v>
@@ -4609,13 +4606,13 @@
         <v>166</v>
       </c>
       <c r="B167" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="C167" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="D167" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="F167" t="s">
         <v>17</v>
@@ -4626,10 +4623,10 @@
         <v>167</v>
       </c>
       <c r="B168" t="s">
+        <v>315</v>
+      </c>
+      <c r="C168" t="s">
         <v>316</v>
-      </c>
-      <c r="C168" t="s">
-        <v>317</v>
       </c>
       <c r="F168" t="s">
         <v>13</v>
@@ -4640,13 +4637,13 @@
         <v>168</v>
       </c>
       <c r="B169" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="C169" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="D169" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="F169" t="s">
         <v>17</v>
@@ -4657,10 +4654,10 @@
         <v>169</v>
       </c>
       <c r="B170" t="s">
+        <v>318</v>
+      </c>
+      <c r="C170" t="s">
         <v>319</v>
-      </c>
-      <c r="C170" t="s">
-        <v>320</v>
       </c>
       <c r="F170" t="s">
         <v>13</v>
@@ -4671,13 +4668,13 @@
         <v>170</v>
       </c>
       <c r="B171" t="s">
+        <v>320</v>
+      </c>
+      <c r="C171" t="s">
+        <v>319</v>
+      </c>
+      <c r="D171" t="s">
         <v>321</v>
-      </c>
-      <c r="C171" t="s">
-        <v>320</v>
-      </c>
-      <c r="D171" t="s">
-        <v>322</v>
       </c>
       <c r="F171" t="s">
         <v>17</v>
@@ -4688,19 +4685,19 @@
         <v>171</v>
       </c>
       <c r="B172" t="s">
+        <v>322</v>
+      </c>
+      <c r="C172" t="s">
+        <v>319</v>
+      </c>
+      <c r="D172" t="s">
         <v>323</v>
       </c>
-      <c r="C172" t="s">
-        <v>320</v>
-      </c>
-      <c r="D172" t="s">
+      <c r="F172" t="s">
+        <v>52</v>
+      </c>
+      <c r="K172" t="s">
         <v>324</v>
-      </c>
-      <c r="F172" t="s">
-        <v>53</v>
-      </c>
-      <c r="K172" t="s">
-        <v>325</v>
       </c>
     </row>
     <row r="173" spans="1:11" x14ac:dyDescent="0.25">
@@ -4708,19 +4705,19 @@
         <v>172</v>
       </c>
       <c r="B173" t="s">
+        <v>325</v>
+      </c>
+      <c r="C173" t="s">
+        <v>319</v>
+      </c>
+      <c r="D173" t="s">
+        <v>166</v>
+      </c>
+      <c r="F173" t="s">
+        <v>52</v>
+      </c>
+      <c r="K173" t="s">
         <v>326</v>
-      </c>
-      <c r="C173" t="s">
-        <v>320</v>
-      </c>
-      <c r="D173" t="s">
-        <v>167</v>
-      </c>
-      <c r="F173" t="s">
-        <v>53</v>
-      </c>
-      <c r="K173" t="s">
-        <v>327</v>
       </c>
     </row>
     <row r="174" spans="1:11" x14ac:dyDescent="0.25">
@@ -4728,13 +4725,13 @@
         <v>173</v>
       </c>
       <c r="B174" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="C174" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="D174" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="F174" t="s">
         <v>17</v>
@@ -4745,10 +4742,10 @@
         <v>174</v>
       </c>
       <c r="B175" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="C175" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="F175" t="s">
         <v>13</v>
@@ -4759,19 +4756,19 @@
         <v>175</v>
       </c>
       <c r="B176" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="C176" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="D176" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="F176" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="G176" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="H176" t="b">
         <v>1</v>
@@ -4782,7 +4779,7 @@
         <v>176</v>
       </c>
       <c r="B177" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="F177" t="s">
         <v>14</v>
@@ -4796,13 +4793,13 @@
         <v>177</v>
       </c>
       <c r="B178" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="C178" t="s">
         <v>12</v>
       </c>
       <c r="D178" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="F178" t="s">
         <v>17</v>
@@ -4813,13 +4810,13 @@
         <v>178</v>
       </c>
       <c r="B179" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="C179" t="s">
         <v>12</v>
       </c>
       <c r="D179" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="F179" t="s">
         <v>17</v>
@@ -4881,144 +4878,144 @@
   <sheetData>
     <row r="1" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="Q1" s="1" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="R1" s="1" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="S1" s="1" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="T1" s="1" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="U1" s="1" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="V1" s="1" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="W1" s="1" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="X1" s="1" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="Y1" s="1" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="Z1" s="1" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="AA1" s="1" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="AB1" s="1" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="AC1" s="1" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="AD1" s="1" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="AE1" s="1" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="AF1" s="1" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="AG1" s="1" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="AH1" s="1" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="AI1" s="1" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="AJ1" s="1" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="AK1" s="1" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="AL1" s="1" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="AM1" s="1" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="AN1" s="1" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="AO1" s="1" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="AP1" s="1" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="2" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>335</v>
+      </c>
+      <c r="B2" t="s">
         <v>336</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
         <v>337</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>338</v>
-      </c>
-      <c r="D2" t="s">
-        <v>339</v>
       </c>
       <c r="E2">
         <v>2012345678</v>
@@ -5027,112 +5024,112 @@
         <v>7712345678</v>
       </c>
       <c r="G2" t="s">
+        <v>339</v>
+      </c>
+      <c r="H2" t="s">
         <v>340</v>
       </c>
-      <c r="H2" t="s">
+      <c r="I2" t="s">
         <v>341</v>
       </c>
-      <c r="I2" t="s">
+      <c r="J2" t="s">
         <v>342</v>
       </c>
-      <c r="J2" t="s">
+      <c r="K2" t="s">
         <v>343</v>
       </c>
-      <c r="K2" t="s">
+      <c r="L2" t="s">
+        <v>343</v>
+      </c>
+      <c r="M2" t="s">
+        <v>343</v>
+      </c>
+      <c r="N2" t="s">
         <v>344</v>
       </c>
-      <c r="L2" t="s">
-        <v>344</v>
-      </c>
-      <c r="M2" t="s">
-        <v>344</v>
-      </c>
-      <c r="N2" t="s">
+      <c r="O2" t="s">
         <v>345</v>
       </c>
-      <c r="O2" t="s">
+      <c r="P2" t="s">
         <v>346</v>
       </c>
-      <c r="P2" t="s">
+      <c r="Q2" t="s">
         <v>347</v>
       </c>
-      <c r="Q2" t="s">
+      <c r="R2" t="s">
         <v>348</v>
       </c>
-      <c r="R2" t="s">
+      <c r="S2" t="s">
         <v>349</v>
       </c>
-      <c r="S2" t="s">
+      <c r="T2" t="s">
         <v>350</v>
       </c>
-      <c r="T2" t="s">
+      <c r="U2" t="s">
+        <v>350</v>
+      </c>
+      <c r="V2" t="s">
+        <v>346</v>
+      </c>
+      <c r="W2" t="s">
         <v>351</v>
       </c>
-      <c r="U2" t="s">
-        <v>351</v>
-      </c>
-      <c r="V2" t="s">
+      <c r="X2" t="s">
         <v>347</v>
       </c>
-      <c r="W2" t="s">
+      <c r="Y2" t="s">
         <v>352</v>
-      </c>
-      <c r="X2" t="s">
-        <v>348</v>
-      </c>
-      <c r="Y2" t="s">
-        <v>353</v>
       </c>
       <c r="Z2" s="2">
         <v>46028</v>
       </c>
       <c r="AA2" t="s">
+        <v>353</v>
+      </c>
+      <c r="AB2" t="s">
+        <v>347</v>
+      </c>
+      <c r="AC2" t="s">
+        <v>352</v>
+      </c>
+      <c r="AD2" t="s">
+        <v>347</v>
+      </c>
+      <c r="AE2" t="s">
+        <v>349</v>
+      </c>
+      <c r="AF2" t="s">
         <v>354</v>
       </c>
-      <c r="AB2" t="s">
-        <v>348</v>
-      </c>
-      <c r="AC2" t="s">
-        <v>353</v>
-      </c>
-      <c r="AD2" t="s">
-        <v>348</v>
-      </c>
-      <c r="AE2" t="s">
-        <v>350</v>
-      </c>
-      <c r="AF2" t="s">
+      <c r="AG2" t="s">
         <v>355</v>
       </c>
-      <c r="AG2" t="s">
-        <v>356</v>
-      </c>
       <c r="AH2" t="s">
+        <v>354</v>
+      </c>
+      <c r="AI2" t="s">
         <v>355</v>
-      </c>
-      <c r="AI2" t="s">
-        <v>356</v>
       </c>
       <c r="AJ2" s="2">
         <v>46029</v>
       </c>
       <c r="AK2" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="AL2" s="2">
         <v>46030</v>
       </c>
       <c r="AM2" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="AN2">
         <v>2</v>
       </c>
       <c r="AO2" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="AP2" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
     </row>
   </sheetData>
@@ -5151,71 +5148,71 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>356</v>
+      </c>
+      <c r="B1" s="3" t="s">
         <v>357</v>
-      </c>
-      <c r="B1" s="3" t="s">
-        <v>358</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>358</v>
+      </c>
+      <c r="B2" s="4" t="s">
         <v>359</v>
-      </c>
-      <c r="B2" s="4" t="s">
-        <v>360</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>360</v>
+      </c>
+      <c r="B3" s="4" t="s">
         <v>361</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>362</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>362</v>
+      </c>
+      <c r="B4" s="4" t="s">
         <v>363</v>
-      </c>
-      <c r="B4" s="4" t="s">
-        <v>364</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="45" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>364</v>
+      </c>
+      <c r="B5" s="4" t="s">
         <v>365</v>
-      </c>
-      <c r="B5" s="4" t="s">
-        <v>366</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
+        <v>366</v>
+      </c>
+      <c r="B6" s="4" t="s">
         <v>367</v>
-      </c>
-      <c r="B6" s="4" t="s">
-        <v>368</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
+        <v>368</v>
+      </c>
+      <c r="B7" s="4" t="s">
         <v>369</v>
-      </c>
-      <c r="B7" s="4" t="s">
-        <v>370</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
+        <v>370</v>
+      </c>
+      <c r="B8" s="4" t="s">
         <v>371</v>
-      </c>
-      <c r="B8" s="4" t="s">
-        <v>372</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="B9" s="4">
         <v>178</v>
@@ -5223,7 +5220,7 @@
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="B10" s="4">
         <v>22</v>
@@ -5231,7 +5228,7 @@
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="B11" s="4">
         <v>55</v>
@@ -5239,15 +5236,15 @@
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
+        <v>375</v>
+      </c>
+      <c r="B12" s="4" t="s">
         <v>376</v>
-      </c>
-      <c r="B12" s="4" t="s">
-        <v>377</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="B13" s="5">
         <v>46147</v>
@@ -5255,7 +5252,7 @@
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="B14" s="5">
         <v>46147</v>
@@ -5263,31 +5260,31 @@
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
+        <v>379</v>
+      </c>
+      <c r="B15" s="4" t="s">
         <v>380</v>
-      </c>
-      <c r="B15" s="4" t="s">
-        <v>381</v>
       </c>
     </row>
     <row r="16" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
+        <v>381</v>
+      </c>
+      <c r="B16" s="4" t="s">
         <v>382</v>
-      </c>
-      <c r="B16" s="4" t="s">
-        <v>383</v>
       </c>
     </row>
     <row r="17" spans="1:2" ht="165" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
+        <v>383</v>
+      </c>
+      <c r="B17" s="4" t="s">
         <v>384</v>
-      </c>
-      <c r="B17" s="4" t="s">
-        <v>385</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="B18" s="4">
         <v>9</v>
@@ -5295,18 +5292,18 @@
     </row>
     <row r="19" spans="1:2" ht="120" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
+        <v>386</v>
+      </c>
+      <c r="B19" s="4" t="s">
         <v>387</v>
-      </c>
-      <c r="B19" s="4" t="s">
-        <v>388</v>
       </c>
     </row>
     <row r="20" spans="1:2" ht="45" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
+        <v>388</v>
+      </c>
+      <c r="B20" s="4" t="s">
         <v>389</v>
-      </c>
-      <c r="B20" s="4" t="s">
-        <v>390</v>
       </c>
     </row>
   </sheetData>
@@ -5326,13 +5323,13 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>390</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>364</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>391</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>365</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>392</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
@@ -5340,54 +5337,54 @@
         <v>26</v>
       </c>
       <c r="B2" t="s">
+        <v>392</v>
+      </c>
+      <c r="C2" t="s">
         <v>393</v>
-      </c>
-      <c r="C2" t="s">
-        <v>394</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B3" t="s">
+        <v>394</v>
+      </c>
+      <c r="C3" t="s">
         <v>395</v>
-      </c>
-      <c r="C3" t="s">
-        <v>396</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B4" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="C4" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>397</v>
+      </c>
+      <c r="B5" t="s">
         <v>398</v>
       </c>
-      <c r="B5" t="s">
+      <c r="C5" t="s">
         <v>399</v>
-      </c>
-      <c r="C5" t="s">
-        <v>400</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
+        <v>400</v>
+      </c>
+      <c r="B6" t="s">
         <v>401</v>
       </c>
-      <c r="B6" t="s">
-        <v>402</v>
-      </c>
       <c r="C6" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: standardize adaptive registration launch
</commit_message>
<xml_diff>
--- a/lorenzo-playwright-kdf/excelFramework/testcases/APE/LSTP_APE_WF001.xlsx
+++ b/lorenzo-playwright-kdf/excelFramework/testcases/APE/LSTP_APE_WF001.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bkrishnan6\ORBIS PAS UKI-LZO\lorenzo-playwright-kdf\excelFramework\testcases\APE\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FBE6BDE1-9A1A-4410-9AEE-E62AA2D73DD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E09B8669-F603-4B79-934B-D3F481A46AA9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{52C8395E-6A7C-4340-B875-65EC1239B4FD}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{52C8395E-6A7C-4340-B875-65EC1239B4FD}"/>
   </bookViews>
   <sheets>
     <sheet name="TestExecution" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1041" uniqueCount="414">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1041" uniqueCount="415">
   <si>
     <t>StepNo</t>
   </si>
@@ -1281,6 +1281,9 @@
   </si>
   <si>
     <t>Create access plan entry</t>
+  </si>
+  <si>
+    <t>launchRegistration</t>
   </si>
 </sst>
 </file>
@@ -2353,7 +2356,7 @@
       </c>
       <c r="E19" s="6"/>
       <c r="F19" s="8" t="s">
-        <v>16</v>
+        <v>414</v>
       </c>
       <c r="G19" s="6"/>
       <c r="H19" s="6"/>
@@ -2479,7 +2482,7 @@
         <v>274</v>
       </c>
       <c r="F23" s="6" t="s">
-        <v>16</v>
+        <v>414</v>
       </c>
       <c r="G23" s="6" t="s">
         <v>274</v>

</xml_diff>